<commit_message>
E-A chiuso: matrici rigenerate, STATO ed ESPERIMENTI aggiornati
RQ1. Lo sweep di epsilon in 2-16 (E-A) ha 19 run valide su 20: a epsilon = 2
il seed 789 non ha attacchi per un errore d'ambiente (segnalazione 42) e va
rilanciato. Attacchi aggregati al caso in tutte le celle; costo oltre soglia
a epsilon <= 8; a epsilon = 16 il costo e' 2.3 volte il no-DP della campagna
ma 3.7 volte nodp-sweep2 appaiato per seed, e la scelta del riferimento resta
da decidere (STATO 3.8). genera_matrici_faseA.py non duplica piu' i fogli
(segnalazione 43); il foglio Utility_privacy_limite mescola pilota, NVFlare e
sweep ripetuti (segnalazione 44, aperta). Include anche il lavoro del
2026-09-22 non ancora committato: decisioni di ESPERIMENTI sez. 0 nella
scheda, fix della segnalazione 37, segnalazione 41, voci di SprintLog.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AM8cmwrGuYL2jwRuBHBhk1
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -561,7 +561,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>136 run in regime naturale</t>
+          <t>156 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="3" ht="160" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>237 run totali</t>
+          <t>257 run totali</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>237 run totali</t>
+          <t>257 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="6" ht="160" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>101 run canary (10 verificate, 16 incompleta)</t>
+          <t>101 run canary (10 verificate, 17 incompleta)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Il controllo positivo e' superato e il negativo bilanciato regge (30/30 round sopra 0.5, min 0.6125, t(4)=9.90 appaiato sui 5 seed). Ma 16 run canary hanno il blocco 'canary' NON registrato nel config: k, duplicati e swap_assignment non sono leggibili dal file, quindi non si puo' stabilire dal JSON se quei bracci di scambio fossero bilanciati. Nessuna e' marcata 'invalidata' proprio per questo: invalidare richiederebbe un'analogia, che la guida vieta.</t>
+          <t>Il controllo positivo e' superato e il negativo bilanciato regge (30/30 round sopra 0.5, min 0.6125, t(4)=9.90 appaiato sui 5 seed). Ma 17 run canary hanno il blocco 'canary' NON registrato nel config: k, duplicati e swap_assignment non sono leggibili dal file, quindi non si puo' stabilire dal JSON se quei bracci di scambio fossero bilanciati. Nessuna e' marcata 'invalidata' proprio per questo: invalidare richiederebbe un'analogia, che la guida vieta.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F134"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3801,12 +3801,12 @@
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -3815,24 +3815,24 @@
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.22936</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="112" ht="18" customHeight="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -3841,24 +3841,24 @@
         </is>
       </c>
       <c r="D112" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.259868</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -3867,24 +3867,24 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.403398</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -3896,7 +3896,7 @@
         <v>10</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.368463</v>
       </c>
       <c r="F114" s="3" t="n">
         <v>25200</v>
@@ -3905,12 +3905,12 @@
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -3922,7 +3922,7 @@
         <v>10</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.378646</v>
       </c>
       <c r="F115" s="3" t="n">
         <v>26829</v>
@@ -3931,12 +3931,12 @@
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -3948,7 +3948,7 @@
         <v>10</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.373247</v>
       </c>
       <c r="F116" s="3" t="n">
         <v>1341</v>
@@ -3957,12 +3957,12 @@
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -3974,7 +3974,7 @@
         <v>10</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.367252</v>
       </c>
       <c r="F117" s="3" t="n">
         <v>25200</v>
@@ -3983,12 +3983,12 @@
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -4000,7 +4000,7 @@
         <v>10</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.377587</v>
       </c>
       <c r="F118" s="3" t="n">
         <v>26829</v>
@@ -4009,12 +4009,12 @@
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4026,7 +4026,7 @@
         <v>10</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.369278</v>
       </c>
       <c r="F119" s="3" t="n">
         <v>1341</v>
@@ -4035,12 +4035,12 @@
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -4049,10 +4049,10 @@
         </is>
       </c>
       <c r="D120" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F120" s="3" t="n">
         <v>25200</v>
@@ -4061,12 +4061,12 @@
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -4075,10 +4075,10 @@
         </is>
       </c>
       <c r="D121" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F121" s="3" t="n">
         <v>26829</v>
@@ -4087,12 +4087,12 @@
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -4101,10 +4101,10 @@
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F122" s="3" t="n">
         <v>1341</v>
@@ -4113,7 +4113,7 @@
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -4127,10 +4127,10 @@
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F123" s="3" t="n">
         <v>25200</v>
@@ -4139,7 +4139,7 @@
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -4153,10 +4153,10 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F124" s="3" t="n">
         <v>26829</v>
@@ -4165,7 +4165,7 @@
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -4179,10 +4179,10 @@
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F125" s="3" t="n">
         <v>1341</v>
@@ -4191,12 +4191,12 @@
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -4208,7 +4208,7 @@
         <v>3</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F126" s="3" t="n">
         <v>25200</v>
@@ -4217,12 +4217,12 @@
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -4234,7 +4234,7 @@
         <v>3</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F127" s="3" t="n">
         <v>26829</v>
@@ -4243,12 +4243,12 @@
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -4260,7 +4260,7 @@
         <v>3</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F128" s="3" t="n">
         <v>1341</v>
@@ -4269,7 +4269,7 @@
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -4295,7 +4295,7 @@
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -4321,7 +4321,7 @@
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -4347,12 +4347,12 @@
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -4364,7 +4364,7 @@
         <v>3</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F132" s="3" t="n">
         <v>25200</v>
@@ -4373,12 +4373,12 @@
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -4390,7 +4390,7 @@
         <v>3</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F133" s="3" t="n">
         <v>26829</v>
@@ -4399,26 +4399,182 @@
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr">
         <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E134" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F134" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E135" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F135" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E136" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F136" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E137" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F137" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="138" ht="18" customHeight="1">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
           <t>verify-sigma-fix.log</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr">
-        <is>
-          <t>no-DP</t>
-        </is>
-      </c>
-      <c r="C134" s="3" t="inlineStr">
-        <is>
-          <t>office1</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E134" s="3" t="n">
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F138" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="139" ht="18" customHeight="1">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E139" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F139" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E140" s="3" t="n">
         <v>0.006995</v>
       </c>
-      <c r="F134" s="3" t="n">
+      <c r="F140" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -4433,7 +4589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4675,28 +4831,28 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.006887</v>
+        <v>0.006265</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.5011</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.5008</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.501</v>
+        <v>0.4999</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.5029</v>
+        <v>0.4998</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0</v>
+        <v>0.0097</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>16</v>
@@ -4723,28 +4879,28 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.012497</v>
+        <v>0.056644</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>4.6</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.4983</v>
+        <v>0.4998</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.4997</v>
+        <v>0.5001</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.4984</v>
+        <v>0.4995</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.4985</v>
+        <v>0.4979</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
+        <v>0.0101</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>8</v>
@@ -4767,92 +4923,92 @@
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=1.0</t>
+          <t>dp-fedavg eps=4.0</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.344612</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>127.9</v>
+        <v>0.127821</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>47.5</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.4999</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.4996</v>
+        <v>0.5002</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.4991</v>
+        <v>0.4988</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.4975</v>
+        <v>0.4959</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.0104</v>
+        <v>0.0092</v>
       </c>
       <c r="J7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="L7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>0.999909</v>
-      </c>
       <c r="M7" s="3" t="n">
-        <v>0.999955</v>
+        <v>1</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+          <t>bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=0.5</t>
+          <t>dp-fedavg eps=2.0</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.422867</v>
+        <v>0.284881</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>157</v>
+        <v>105.8</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.5</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.5001</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.4988</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.4978</v>
+        <v>0.4952</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.0098</v>
+        <v>0.0094</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.986614</v>
+        <v>1</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0.9933070000000001</v>
+        <v>1</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
@@ -4863,44 +5019,44 @@
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=0.1</t>
+          <t>dp-fedavg eps=1.0</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.422351</v>
+        <v>0.344612</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>156.8</v>
+        <v>127.9</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>0.4995</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.4996</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4991</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.4991</v>
+        <v>0.4975</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0104</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0.462117</v>
+        <v>0.999909</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>0.731059</v>
+        <v>0.999955</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
@@ -4911,44 +5067,44 @@
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>local eps=1.0</t>
+          <t>dp-fedavg eps=0.5</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.375652</v>
+        <v>0.422867</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>139.5</v>
+        <v>157</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.4996</v>
+        <v>0.4998</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.4993</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.4992</v>
+        <v>0.4994</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.4984</v>
+        <v>0.4978</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.0108</v>
+        <v>0.0098</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.999909</v>
+        <v>0.986614</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>0.999955</v>
+        <v>0.9933070000000001</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
@@ -4959,44 +5115,44 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>local eps=0.5</t>
+          <t>dp-fedavg eps=0.1</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.423458</v>
+        <v>0.422351</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>157.2</v>
+        <v>156.8</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4995</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>0.4994</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.4996</v>
+        <v>0.4998</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.4983</v>
+        <v>0.4991</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.986614</v>
+        <v>0.462117</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.9933070000000001</v>
+        <v>0.731059</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
@@ -5007,44 +5163,44 @@
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>local eps=0.1</t>
+          <t>local eps=1.0</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.4157</v>
+        <v>0.375652</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>154.3</v>
+        <v>139.5</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.4999</v>
+        <v>0.4996</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.4997</v>
+        <v>0.4995</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.4997</v>
+        <v>0.4992</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.4986</v>
+        <v>0.4984</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0108</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.462117</v>
+        <v>0.999909</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.731059</v>
+        <v>0.999955</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
@@ -5055,38 +5211,134 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>local eps=0.5</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.411787</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>152.9</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.4998</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.4995</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.4997</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.4978</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.0106</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>0.986614</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>0.9933070000000001</v>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>local eps=0.1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.419873</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.4993</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.4992</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.4998</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.4987</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0.462117</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0.731059</v>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C15" s="3" t="n">
         <v>0.002693</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E15" s="3" t="n">
         <v>0.5027</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F15" s="3" t="n">
         <v>0.5011</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="G15" s="3" t="n">
         <v>0.5096000000000001</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H15" s="3" t="n">
         <v>0.5129</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I15" s="3" t="n">
         <v>0.0098</v>
       </c>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="n"/>
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>riferimento senza DP: nessuna garanzia da confrontare</t>
         </is>

</xml_diff>

<commit_message>
RQ1: costo su holdout del modello rilasciato (seg 46), test appaiato per record (seg 47), accountant record-DP con limite shuffle (seg 4), common_init (seg 48), norm group sotto record-DP (seg 49), log norme dei delta; matrici e STATO rigenerati
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -561,7 +561,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>156 run in regime naturale</t>
+          <t>157 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="3" ht="160" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>257 run totali</t>
+          <t>258 run totali</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>257 run totali</t>
+          <t>258 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -955,7 +955,7 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>loss finale</t>
+          <t>loss addestramento locale (ultimo round)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -3619,7 +3619,7 @@
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>rdp_e1000_s5.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -3629,23 +3629,23 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>0.004526</v>
+        <v>0.001897</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>rdp_eps_sweep.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -3655,28 +3655,28 @@
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>0.003026</v>
+        <v>0.001957</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>recorddp_fast_s42.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -3685,19 +3685,19 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.005368</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>recorddp_pair_s42.log</t>
+          <t>rdp_e1000_s5.log</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3714,7 +3714,7 @@
         <v>3</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>0.000301</v>
+        <v>0.004526</v>
       </c>
       <c r="F107" s="3" t="n">
         <v>1924</v>
@@ -3723,12 +3723,12 @@
     <row r="108" ht="18" customHeight="1">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>recorddp_smoke.log</t>
+          <t>rdp_eps_sweep.log</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -3740,7 +3740,7 @@
         <v>3</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.003026</v>
       </c>
       <c r="F108" s="3" t="n">
         <v>1924</v>
@@ -3749,12 +3749,12 @@
     <row r="109" ht="18" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>recorddp_swap_s42.log</t>
+          <t>recorddp_fast_s42.log</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -3766,7 +3766,7 @@
         <v>3</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>0.000237</v>
+        <v>0.288884</v>
       </c>
       <c r="F109" s="3" t="n">
         <v>1924</v>
@@ -3775,7 +3775,7 @@
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>ref_e1000_group.log</t>
+          <t>recorddp_pair_s42.log</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3792,7 +3792,7 @@
         <v>3</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>2.6e-05</v>
+        <v>0.000301</v>
       </c>
       <c r="F110" s="3" t="n">
         <v>1924</v>
@@ -3801,64 +3801,64 @@
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>recorddp_smoke.log</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.22936</v>
+        <v>0.288884</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>25143</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="112" ht="18" customHeight="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>recorddp_swap_s42.log</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D112" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.259868</v>
+        <v>0.000237</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>26892</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>ref_e1000_group.log</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -3867,19 +3867,19 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>0.403398</v>
+        <v>2.6e-05</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -3896,16 +3896,16 @@
         <v>10</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.368463</v>
+        <v>0.211667</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3922,16 +3922,16 @@
         <v>10</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.378646</v>
+        <v>0.223153</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3948,21 +3948,21 @@
         <v>10</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.373247</v>
+        <v>0.303531</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -3971,24 +3971,24 @@
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.378351</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -3997,24 +3997,24 @@
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.428026</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4023,24 +4023,24 @@
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.395166</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -4052,21 +4052,21 @@
         <v>10</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.211667</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -4078,21 +4078,21 @@
         <v>10</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.223153</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -4104,21 +4104,21 @@
         <v>10</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.303531</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -4130,7 +4130,7 @@
         <v>10</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.368463</v>
       </c>
       <c r="F123" s="3" t="n">
         <v>25200</v>
@@ -4139,12 +4139,12 @@
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -4156,7 +4156,7 @@
         <v>10</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.378646</v>
       </c>
       <c r="F124" s="3" t="n">
         <v>26829</v>
@@ -4165,12 +4165,12 @@
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -4182,7 +4182,7 @@
         <v>10</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.373247</v>
       </c>
       <c r="F125" s="3" t="n">
         <v>1341</v>
@@ -4191,12 +4191,12 @@
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -4205,10 +4205,10 @@
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.367252</v>
       </c>
       <c r="F126" s="3" t="n">
         <v>25200</v>
@@ -4217,12 +4217,12 @@
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -4231,10 +4231,10 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.377587</v>
       </c>
       <c r="F127" s="3" t="n">
         <v>26829</v>
@@ -4243,12 +4243,12 @@
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -4257,10 +4257,10 @@
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.369278</v>
       </c>
       <c r="F128" s="3" t="n">
         <v>1341</v>
@@ -4269,12 +4269,12 @@
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -4283,10 +4283,10 @@
         </is>
       </c>
       <c r="D129" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F129" s="3" t="n">
         <v>25200</v>
@@ -4295,12 +4295,12 @@
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -4309,10 +4309,10 @@
         </is>
       </c>
       <c r="D130" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F130" s="3" t="n">
         <v>26829</v>
@@ -4321,12 +4321,12 @@
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -4335,10 +4335,10 @@
         </is>
       </c>
       <c r="D131" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F131" s="3" t="n">
         <v>1341</v>
@@ -4347,12 +4347,12 @@
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -4361,10 +4361,10 @@
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.002174</v>
       </c>
       <c r="F132" s="3" t="n">
         <v>25200</v>
@@ -4373,12 +4373,12 @@
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -4387,10 +4387,10 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002005</v>
       </c>
       <c r="F133" s="3" t="n">
         <v>26829</v>
@@ -4399,12 +4399,12 @@
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -4413,10 +4413,10 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.005707</v>
       </c>
       <c r="F134" s="3" t="n">
         <v>1341</v>
@@ -4425,7 +4425,7 @@
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -4451,7 +4451,7 @@
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -4477,7 +4477,7 @@
     <row r="137" ht="18" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -4503,7 +4503,7 @@
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4529,7 +4529,7 @@
     <row r="139" ht="18" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4555,7 +4555,7 @@
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -4575,6 +4575,240 @@
         <v>0.006995</v>
       </c>
       <c r="F140" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E141" s="3" t="n">
+        <v>0.086894</v>
+      </c>
+      <c r="F141" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>0.076844</v>
+      </c>
+      <c r="F142" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E143" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F143" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F144" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E145" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F145" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E147" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F147" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F148" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F149" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -4589,23 +4823,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="70" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4621,60 +4856,70 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>loss finale</t>
+          <t>loss holdout modello rilasciato</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>x rispetto a no-DP</t>
+          <t>x rispetto a no-DP (holdout)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>x rispetto a no-DP (locale)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Yeom</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Shadow</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>LiRA</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>LiRA composto</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>TPR@1%FPR</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>eps per round</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>eps_tot (T=10, base)</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Adv max teorica</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>AUC max teorica</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>lettura</t>
         </is>
@@ -4690,41 +4935,47 @@
         <v>14</v>
       </c>
       <c r="C2" s="3" t="n">
+        <v>0.385978</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>158.3</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>0.291187</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="F2" s="3" t="n">
         <v>108.1</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="G2" s="3" t="n">
         <v>0.4997</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>0.4993</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>0.5063</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>0.5027</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>0.0103</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>0.999909</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>0.999955</v>
       </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4738,41 +4989,47 @@
         <v>9</v>
       </c>
       <c r="C3" s="3" t="n">
+        <v>0.454904</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>186.6</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>0.474589</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="F3" s="3" t="n">
         <v>176.2</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="G3" s="3" t="n">
         <v>0.4991</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>0.4987</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>0.5002</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>0.5016</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>0.0102</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>0.986614</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>0.9933070000000001</v>
       </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4786,41 +5043,47 @@
         <v>5</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.481279</v>
+        <v>0.435625</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>178.7</v>
       </c>
       <c r="E4" s="3" t="n">
+        <v>0.481279</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>178.7</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>0.4992</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="I4" s="3" t="n">
         <v>0.5004999999999999</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>0.502</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="K4" s="3" t="n">
         <v>0.0105</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="L4" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="M4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="N4" s="3" t="n">
         <v>0.462117</v>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="O4" s="3" t="n">
         <v>0.731059</v>
       </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4834,41 +5097,47 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="n">
+        <v>0.115064</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>0.006265</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="F5" s="3" t="n">
         <v>2.3</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="G5" s="3" t="n">
         <v>0.5011</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>0.5008</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="I5" s="3" t="n">
         <v>0.4999</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>0.0097</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="L5" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="M5" s="3" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="N5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="O5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>COSTO OLTRE LA SOGLIA DI 3x (sezione 0 di ESPERIMENTI.md). bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4882,41 +5151,47 @@
         <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
+        <v>0.225233</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>0.056644</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="F6" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="G6" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="H6" s="3" t="n">
         <v>0.5001</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="I6" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>0.4979</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="K6" s="3" t="n">
         <v>0.0101</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="L6" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="M6" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="N6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M6" s="3" t="n">
+      <c r="O6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4930,41 +5205,47 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="n">
+        <v>0.298684</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>0.127821</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="F7" s="3" t="n">
         <v>47.5</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="G7" s="3" t="n">
         <v>0.4999</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="H7" s="3" t="n">
         <v>0.5002</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="I7" s="3" t="n">
         <v>0.4988</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>0.4959</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="K7" s="3" t="n">
         <v>0.0092</v>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="L7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="M7" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="N7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="3" t="n">
+      <c r="O7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -4975,44 +5256,50 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.284881</v>
+        <v>0.365534</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>105.8</v>
+        <v>149.9</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.5</v>
+        <v>0.274026</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.5001</v>
+        <v>101.7</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.4988</v>
+        <v>0.5004</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.4952</v>
+        <v>0.5004999999999999</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.0094</v>
+        <v>0.4989</v>
       </c>
       <c r="J8" s="3" t="n">
+        <v>0.4957</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="L8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="M8" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="L8" s="3" t="n">
+      <c r="N8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M8" s="3" t="n">
+      <c r="O8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5026,41 +5313,47 @@
         <v>14</v>
       </c>
       <c r="C9" s="3" t="n">
+        <v>0.39186</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>160.7</v>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>0.344612</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="F9" s="3" t="n">
         <v>127.9</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="G9" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="H9" s="3" t="n">
         <v>0.4996</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="I9" s="3" t="n">
         <v>0.4991</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="J9" s="3" t="n">
         <v>0.4975</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="K9" s="3" t="n">
         <v>0.0104</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="L9" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="M9" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="L9" s="3" t="n">
+      <c r="N9" s="3" t="n">
         <v>0.999909</v>
       </c>
-      <c r="M9" s="3" t="n">
+      <c r="O9" s="3" t="n">
         <v>0.999955</v>
       </c>
-      <c r="N9" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5074,41 +5367,47 @@
         <v>10</v>
       </c>
       <c r="C10" s="3" t="n">
+        <v>0.407656</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>167.2</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>0.422867</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="F10" s="3" t="n">
         <v>157</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="G10" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="H10" s="3" t="n">
         <v>0.4993</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="I10" s="3" t="n">
         <v>0.4994</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="J10" s="3" t="n">
         <v>0.4978</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="K10" s="3" t="n">
         <v>0.0098</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="L10" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="K10" s="3" t="n">
+      <c r="M10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L10" s="3" t="n">
+      <c r="N10" s="3" t="n">
         <v>0.986614</v>
       </c>
-      <c r="M10" s="3" t="n">
+      <c r="O10" s="3" t="n">
         <v>0.9933070000000001</v>
       </c>
-      <c r="N10" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5122,41 +5421,47 @@
         <v>10</v>
       </c>
       <c r="C11" s="3" t="n">
+        <v>0.422825</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>173.4</v>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>0.422351</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="F11" s="3" t="n">
         <v>156.8</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="G11" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="H11" s="3" t="n">
         <v>0.4994</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="I11" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>0.4991</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="K11" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="L11" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="K11" s="3" t="n">
+      <c r="M11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="3" t="n">
+      <c r="N11" s="3" t="n">
         <v>0.462117</v>
       </c>
-      <c r="M11" s="3" t="n">
+      <c r="O11" s="3" t="n">
         <v>0.731059</v>
       </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5170,41 +5475,47 @@
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
+        <v>0.384188</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>157.6</v>
+      </c>
+      <c r="E12" s="3" t="n">
         <v>0.375652</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="F12" s="3" t="n">
         <v>139.5</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="G12" s="3" t="n">
         <v>0.4996</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="H12" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="I12" s="3" t="n">
         <v>0.4992</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="J12" s="3" t="n">
         <v>0.4984</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="K12" s="3" t="n">
         <v>0.0108</v>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="L12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="3" t="n">
+      <c r="M12" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="L12" s="3" t="n">
+      <c r="N12" s="3" t="n">
         <v>0.999909</v>
       </c>
-      <c r="M12" s="3" t="n">
+      <c r="O12" s="3" t="n">
         <v>0.999955</v>
       </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5218,41 +5529,47 @@
         <v>6</v>
       </c>
       <c r="C13" s="3" t="n">
+        <v>0.397979</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>0.411787</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="F13" s="3" t="n">
         <v>152.9</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="G13" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="H13" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="I13" s="3" t="n">
         <v>0.4997</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="J13" s="3" t="n">
         <v>0.4978</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="K13" s="3" t="n">
         <v>0.0106</v>
       </c>
-      <c r="J13" s="3" t="n">
+      <c r="L13" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="K13" s="3" t="n">
+      <c r="M13" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="L13" s="3" t="n">
+      <c r="N13" s="3" t="n">
         <v>0.986614</v>
       </c>
-      <c r="M13" s="3" t="n">
+      <c r="O13" s="3" t="n">
         <v>0.9933070000000001</v>
       </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5266,41 +5583,47 @@
         <v>6</v>
       </c>
       <c r="C14" s="3" t="n">
+        <v>0.422283</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>173.2</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>0.419873</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="F14" s="3" t="n">
         <v>155.9</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="G14" s="3" t="n">
         <v>0.4993</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="H14" s="3" t="n">
         <v>0.4992</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="I14" s="3" t="n">
         <v>0.4998</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="J14" s="3" t="n">
         <v>0.4987</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="K14" s="3" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="J14" s="3" t="n">
+      <c r="L14" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="K14" s="3" t="n">
+      <c r="M14" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="3" t="n">
+      <c r="N14" s="3" t="n">
         <v>0.462117</v>
       </c>
-      <c r="M14" s="3" t="n">
+      <c r="O14" s="3" t="n">
         <v>0.731059</v>
       </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>UTILITY DISTRUTTA (loss oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
@@ -5314,31 +5637,37 @@
         <v>49</v>
       </c>
       <c r="C15" s="3" t="n">
+        <v>0.002438</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>0.002693</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="F15" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="G15" s="3" t="n">
         <v>0.5027</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="H15" s="3" t="n">
         <v>0.5011</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="I15" s="3" t="n">
         <v>0.5096000000000001</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="J15" s="3" t="n">
         <v>0.5129</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="K15" s="3" t="n">
         <v>0.0098</v>
       </c>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="n"/>
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>riferimento senza DP: nessuna garanzia da confrontare</t>
         </is>
@@ -5355,7 +5684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5364,10 +5693,15 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="80" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="80" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5388,7 +5722,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>record segnalati</t>
+          <t>record segnalati (membri)</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -5403,20 +5737,45 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>z</t>
+          <t>z membri (stabilita' del ranking)</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
+          <t>z non-membri (controllo)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>z membri meno non-membri</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>test appaiato: diff. media di percentile (membro - non membro)</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>errore standard</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>z appaiato</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
           <t>% osservata</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>% attesa</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>lettura</t>
         </is>
@@ -5443,25 +5802,40 @@
       <c r="F2" s="3" t="n">
         <v>16.15</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="3" t="n">
         <v>7.559</v>
       </c>
       <c r="H2" s="3" t="n">
+        <v>6.854</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.0561</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>2.346</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>1.651</v>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>ECCESSO REALE: esiste un sottoinsieme di record sistematicamente nel decile alto su seed indipendenti. Invisibile nell'AUC aggregata, che in questa cella e' ~0.51.</t>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="76" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg_eps1</t>
+          <t>dp-fedavg_eps16</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -5471,33 +5845,48 @@
         <v>17561</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>290</v>
+        <v>326</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>289.75</v>
+        <v>290.44</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>15.88</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>0.016</v>
+        <v>16.76</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2.121</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.651</v>
+        <v>0.224</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>indistinguibile dal caso. ATTENZIONE: in questa cella l'utility e' distrutta (loss oltre 100x), quindi l'assenza di eccesso NON prova che la DP protegga: un modello che non impara non espone.</t>
+        <v>1.43</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.0692</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0.2215</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.312</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>1.856</v>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>1.654</v>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="76" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>central_eps1</t>
+          <t>dp-fedavg_eps8</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -5507,33 +5896,48 @@
         <v>17561</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>289.9</v>
+        <v>291.5</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>14.74</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>0.617</v>
+        <v>16.55</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.091</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.703</v>
+        <v>3.451</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.651</v>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>indistinguibile dal caso. ATTENZIONE: in questa cella l'utility e' distrutta (loss oltre 100x), quindi l'assenza di eccesso NON prova che la DP protegga: un modello che non impara non espone.</t>
+        <v>-2.275</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.1222</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.2202</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="76" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>local_eps1</t>
+          <t>dp-fedavg_eps4</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -5543,33 +5947,252 @@
         <v>17561</v>
       </c>
       <c r="D5" s="3" t="n">
+        <v>355</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>288.94</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>4.308</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3.864</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>-0.3059</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0.2212</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>-1.383</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>2.022</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>1.645</v>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="76" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>dp-fedavg_eps2</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>337</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>290.26</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>2.878</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>2.705</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>-0.2964</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.2213</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>-1.339</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>1.919</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>1.653</v>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="76" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>dp-fedavg_eps1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>290</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>289.75</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>-0.413</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>-0.2067</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>-0.9350000000000001</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>1.651</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="76" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>central_eps1</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>299</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>289.9</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1.912</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>-0.968</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.1989</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.2195</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>1.703</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>1.651</v>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="76" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>local_eps1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D9" s="3" t="n">
         <v>291</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E9" s="3" t="n">
         <v>289.79</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F9" s="3" t="n">
         <v>17.34</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G9" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H9" s="3" t="n">
+        <v>1.528</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>-0.984</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>-0.2905</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0.2208</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>-1.316</v>
+      </c>
+      <c r="M9" s="3" t="n">
         <v>1.657</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="N9" s="3" t="n">
         <v>1.65</v>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>indistinguibile dal caso. ATTENZIONE: in questa cella l'utility e' distrutta (loss oltre 100x), quindi l'assenza di eccesso NON prova che la DP protegga: un modello che non impara non espone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed)</t>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>
       </c>
     </row>
@@ -5584,7 +6207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5705,12 +6328,12 @@
     <row r="5" ht="150" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>x rispetto a no-DP</t>
+          <t>x rispetto a no-DP (holdout)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Rapporto fra la loss finale sull'holdout naturale della cella e quella della cella senza DP. E' la misura di costo.</t>
+          <t>Rapporto fra la loss di ricostruzione sull'holdout naturale del modello globale RILASCIATO all'ultimo round e quella della cella senza DP. E' la misura di costo (soglia di 3x, sezione 0 di ESPERIMENTI.md). Fino al 2026-09-24 la colonna usava la loss di addestramento locale (segnalazione 46).</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -5732,52 +6355,79 @@
     <row r="6" ht="150" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>A0 / A1 / A2 / A3</t>
+          <t>loss addestramento locale (diagnostica)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Punti di osservazione dell'avversario sulla stessa pipeline di privatizzazione. A0 = nessuna DP. A1 = update grezzo g (dp-fedavg). A2 = update clippato (central). A3 = update clippato e rumorizzato (local).</t>
+          <t>Media pesata delle loss di addestramento locale dei client nell'ultimo round, mediata sulle 50 epoche e calcolata prima del rumore DP di quel round (per_round[T].fl.mean_loss; nel log: 'Round T — loss globale').</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Sono ORDINATI per informazione: A2 e A3 si ottengono da A1 con trasformazioni che distruggono informazione. Chi osserva A1 puo' calcolarsi A2 e A3; il contrario e' impossibile. Quindi un nullo ad A1 limita anche gli altri due: non c'era segnale da sopprimere.</t>
+          <t>NON e' la qualita' del modello rilasciato. Senza DP coincide quasi con la loss sull'holdout; con DP client-level misura quanto bene un client riadatta localmente il modello rumoroso che riceve, e la distanza dalla loss sull'holdout misura il danno del rumore aggiunto all'aggregazione.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>registro run, colonna superficie dell'attacco</t>
+          <t>fogli Utility_privacy_limite e Costo_per_sito</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>docs/paper/latex_dsn2027/sections/threat_model.tex</t>
+          <t>segnalazione 46</t>
         </is>
       </c>
     </row>
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>A0 / A1 / A2 / A3</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Punti di osservazione dell'avversario sulla stessa pipeline di privatizzazione. A0 = nessuna DP. A1 = update grezzo g (dp-fedavg). A2 = update clippato (central). A3 = update clippato e rumorizzato (local).</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sono ORDINATI per informazione: A2 e A3 si ottengono da A1 con trasformazioni che distruggono informazione. Chi osserva A1 puo' calcolarsi A2 e A3; il contrario e' impossibile. Quindi un nullo ad A1 limita anche gli altri due: non c'era segnale da sopprimere.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>registro run, colonna superficie dell'attacco</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>docs/paper/latex_dsn2027/sections/threat_model.tex</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>stato di validita'</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>I cinque stati previsti dalla guida: verificata, completata da verificare, invalidata, incompleta, pianificata.</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>'completata da verificare' e' lo stato di default e NON significa sospetta: significa che la tracciabilita' completa richiesta dalla Fase A non e' ricostruibile, perche' commit e hash degli split non erano registrati prima del 2026-09-21.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>registro run</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>ChargeShield_FL_spina_dorsale_consolidata.md riga 150</t>
         </is>

</xml_diff>

<commit_message>
RQ1: etichetta di cella comune (seg 44, 45, 53), matrici ricomposte con riferimento no-DP di 5 run; prova E-B: durata e cartella nuova; SprintLog 10zz+127
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -561,7 +561,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>157 run in regime naturale</t>
+          <t>158 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="3" ht="160" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>258 run totali</t>
+          <t>260 run totali</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>258 run totali</t>
+          <t>260 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="6" ht="160" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>101 run canary (10 verificate, 17 incompleta)</t>
+          <t>101 run canary (10 verificate, 18 incompleta)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Il controllo positivo e' superato e il negativo bilanciato regge (30/30 round sopra 0.5, min 0.6125, t(4)=9.90 appaiato sui 5 seed). Ma 17 run canary hanno il blocco 'canary' NON registrato nel config: k, duplicati e swap_assignment non sono leggibili dal file, quindi non si puo' stabilire dal JSON se quei bracci di scambio fossero bilanciati. Nessuna e' marcata 'invalidata' proprio per questo: invalidare richiederebbe un'analogia, che la guida vieta.</t>
+          <t>Il controllo positivo e' superato e il negativo bilanciato regge (30/30 round sopra 0.5, min 0.6125, t(4)=9.90 appaiato sui 5 seed). Ma 18 run canary hanno il blocco 'canary' NON registrato nel config: k, duplicati e swap_assignment non sono leggibili dal file, quindi non si puo' stabilire dal JSON se quei bracci di scambio fossero bilanciati. Nessuna e' marcata 'invalidata' proprio per questo: invalidare richiederebbe un'analogia, che la guida vieta.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>check_significance.py deduplica per (dp_mode, epsilon, seed) scegliendo il file piu' recente. E' una scelta implicita: va dichiarata nel paper o sostituita con un criterio esplicito.</t>
+          <t>check_significance.py e questo script compongono le celle con la stessa regola (segnalazioni 44, 45, 53, 2026-09-24): etichetta dai campi registrati nel JSON (scripts/etichetta_cella.py), cartelle _*, entity-split*, nvflare-* e fedmia-gradient-* escluse, una run per (cella, seed del config), la piu' recente. La scelta del seed del config invece del nome della cartella va dichiarata (segnalazione 9).</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2553,12 +2553,12 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>diag-eps16-dpfedavg.log</t>
+          <t>ctrl_common_init_s42.log</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=16.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2567,10 +2567,10 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.006589</v>
+        <v>0.001266</v>
       </c>
       <c r="F63" s="3" t="n">
         <v>25200</v>
@@ -2579,12 +2579,12 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>diag-eps16-dpfedavg.log</t>
+          <t>ctrl_common_init_s42.log</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=16.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2593,10 +2593,10 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.007024</v>
+        <v>0.001136</v>
       </c>
       <c r="F64" s="3" t="n">
         <v>26829</v>
@@ -2605,12 +2605,12 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>diag-eps16-dpfedavg.log</t>
+          <t>ctrl_common_init_s42.log</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=16.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2619,10 +2619,10 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.009767</v>
+        <v>0.001967</v>
       </c>
       <c r="F65" s="3" t="n">
         <v>1341</v>
@@ -2631,12 +2631,12 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>diag-eps8-dpfedavg.log</t>
+          <t>ctrl_riproduzione_s42.log</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=8.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2645,10 +2645,10 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.008470999999999999</v>
+        <v>0.002174</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>25200</v>
@@ -2657,12 +2657,12 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>diag-eps8-dpfedavg.log</t>
+          <t>ctrl_riproduzione_s42.log</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=8.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -2671,10 +2671,10 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.0158</v>
+        <v>0.002005</v>
       </c>
       <c r="F67" s="3" t="n">
         <v>26829</v>
@@ -2683,12 +2683,12 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>diag-eps8-dpfedavg.log</t>
+          <t>ctrl_riproduzione_s42.log</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=8.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2697,10 +2697,10 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.022073</v>
+        <v>0.005707</v>
       </c>
       <c r="F68" s="3" t="n">
         <v>1341</v>
@@ -2709,12 +2709,12 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula-central.log</t>
+          <t>diag-eps16-dpfedavg.log</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -2726,7 +2726,7 @@
         <v>3</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.006589</v>
       </c>
       <c r="F69" s="3" t="n">
         <v>25200</v>
@@ -2735,12 +2735,12 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula-central.log</t>
+          <t>diag-eps16-dpfedavg.log</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -2752,7 +2752,7 @@
         <v>3</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.007024</v>
       </c>
       <c r="F70" s="3" t="n">
         <v>26829</v>
@@ -2761,12 +2761,12 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula-central.log</t>
+          <t>diag-eps16-dpfedavg.log</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -2778,7 +2778,7 @@
         <v>3</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.009767</v>
       </c>
       <c r="F71" s="3" t="n">
         <v>1341</v>
@@ -2787,12 +2787,12 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula.log</t>
+          <t>diag-eps8-dpfedavg.log</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=8.0)</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -2804,7 +2804,7 @@
         <v>3</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.008470999999999999</v>
       </c>
       <c r="F72" s="3" t="n">
         <v>25200</v>
@@ -2813,12 +2813,12 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula.log</t>
+          <t>diag-eps8-dpfedavg.log</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=8.0)</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -2830,7 +2830,7 @@
         <v>3</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.0158</v>
       </c>
       <c r="F73" s="3" t="n">
         <v>26829</v>
@@ -2839,12 +2839,12 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>diag-matched-formula.log</t>
+          <t>diag-eps8-dpfedavg.log</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=8.0)</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -2856,7 +2856,7 @@
         <v>3</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.022073</v>
       </c>
       <c r="F74" s="3" t="n">
         <v>1341</v>
@@ -2865,12 +2865,12 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>diag-mu-inversion.log</t>
+          <t>diag-matched-formula-central.log</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -2882,7 +2882,7 @@
         <v>3</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F75" s="3" t="n">
         <v>25200</v>
@@ -2891,12 +2891,12 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>diag-mu-inversion.log</t>
+          <t>diag-matched-formula-central.log</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -2908,7 +2908,7 @@
         <v>3</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F76" s="3" t="n">
         <v>26829</v>
@@ -2917,12 +2917,12 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>diag-mu-inversion.log</t>
+          <t>diag-matched-formula-central.log</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -2934,7 +2934,7 @@
         <v>3</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.120528</v>
       </c>
       <c r="F77" s="3" t="n">
         <v>1341</v>
@@ -2943,7 +2943,7 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>diag-nodp-sigma.log</t>
+          <t>diag-matched-formula.log</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>diag-nodp-sigma.log</t>
+          <t>diag-matched-formula.log</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -2995,7 +2995,7 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>diag-nodp-sigma.log</t>
+          <t>diag-matched-formula.log</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -3021,7 +3021,7 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>diag-persample.log</t>
+          <t>diag-mu-inversion.log</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -3035,10 +3035,10 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>0.00777</v>
+        <v>0.003394</v>
       </c>
       <c r="F81" s="3" t="n">
         <v>25200</v>
@@ -3047,7 +3047,7 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>diag-persample.log</t>
+          <t>diag-mu-inversion.log</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -3061,10 +3061,10 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>0.006383</v>
+        <v>0.002953</v>
       </c>
       <c r="F82" s="3" t="n">
         <v>26829</v>
@@ -3073,7 +3073,7 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>diag-persample.log</t>
+          <t>diag-mu-inversion.log</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -3087,10 +3087,10 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0.010411</v>
+        <v>0.006995</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>1341</v>
@@ -3099,7 +3099,7 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>e100_group_base_s42.log</t>
+          <t>diag-nodp-sigma.log</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -3109,23 +3109,23 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>0.000301</v>
+        <v>0.003394</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke.log</t>
+          <t>diag-nodp-sigma.log</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -3135,23 +3135,23 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>0.007372</v>
+        <v>0.002953</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>25200</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke.log</t>
+          <t>diag-nodp-sigma.log</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -3161,23 +3161,23 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>0.005925</v>
+        <v>0.006995</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>26829</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke.log</t>
+          <t>diag-persample.log</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -3187,23 +3187,23 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>0.012637</v>
+        <v>0.00777</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>1341</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke2.log</t>
+          <t>diag-persample.log</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -3213,23 +3213,23 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>0.007372</v>
+        <v>0.006383</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>25200</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke2.log</t>
+          <t>diag-persample.log</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -3239,23 +3239,23 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>0.005925</v>
+        <v>0.010411</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>26829</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke2.log</t>
+          <t>e100_group_base_s42.log</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -3269,19 +3269,19 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>0.012637</v>
+        <v>0.000301</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>1341</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="91" ht="18" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke4.log</t>
+          <t>fedmia_gradient_smoke.log</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -3307,7 +3307,7 @@
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke4.log</t>
+          <t>fedmia_gradient_smoke.log</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -3333,7 +3333,7 @@
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>fedmia_gradient_smoke4.log</t>
+          <t>fedmia_gradient_smoke.log</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -3359,7 +3359,7 @@
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>final_dsn_batch.log</t>
+          <t>fedmia_gradient_smoke2.log</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -3369,23 +3369,23 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>2.6e-05</v>
+        <v>0.007372</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>full-campaign-20260815.log</t>
+          <t>fedmia_gradient_smoke2.log</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -3395,23 +3395,23 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.005925</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>25200</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>full-campaign-20260815.log</t>
+          <t>fedmia_gradient_smoke2.log</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -3421,23 +3421,23 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.012637</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>26829</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>full-campaign-20260815.log</t>
+          <t>fedmia_gradient_smoke4.log</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -3447,80 +3447,80 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.007372</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>1341</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>local-dp-eps1.0.log</t>
+          <t>fedmia_gradient_smoke4.log</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>0.367528</v>
+        <v>0.005925</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>25200</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>local-dp-eps1.0.log</t>
+          <t>fedmia_gradient_smoke4.log</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>0.377736</v>
+        <v>0.012637</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>26829</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>local-dp-eps1.0.log</t>
+          <t>final_dsn_batch.log</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -3529,19 +3529,19 @@
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>0.371144</v>
+        <v>2.6e-05</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>1341</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>nodp-sweep.log</t>
+          <t>full-campaign-20260815.log</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -3567,7 +3567,7 @@
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>nodp-sweep.log</t>
+          <t>full-campaign-20260815.log</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -3593,7 +3593,7 @@
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>nodp-sweep.log</t>
+          <t>full-campaign-20260815.log</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -3619,12 +3619,12 @@
     <row r="104" ht="18" customHeight="1">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>local-dp-eps1.0.log</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -3636,7 +3636,7 @@
         <v>10</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>0.001897</v>
+        <v>0.367528</v>
       </c>
       <c r="F104" s="3" t="n">
         <v>25200</v>
@@ -3645,12 +3645,12 @@
     <row r="105" ht="18" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>local-dp-eps1.0.log</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -3662,7 +3662,7 @@
         <v>10</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>0.001957</v>
+        <v>0.377736</v>
       </c>
       <c r="F105" s="3" t="n">
         <v>26829</v>
@@ -3671,12 +3671,12 @@
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>local-dp-eps1.0.log</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -3688,7 +3688,7 @@
         <v>10</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>0.005368</v>
+        <v>0.371144</v>
       </c>
       <c r="F106" s="3" t="n">
         <v>1341</v>
@@ -3697,7 +3697,7 @@
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>rdp_e1000_s5.log</t>
+          <t>nodp-sweep.log</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -3707,23 +3707,23 @@
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D107" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>0.004526</v>
+        <v>0.002174</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="108" ht="18" customHeight="1">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>rdp_eps_sweep.log</t>
+          <t>nodp-sweep.log</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -3733,28 +3733,28 @@
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>0.003026</v>
+        <v>0.002005</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="109" ht="18" customHeight="1">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>recorddp_fast_s42.log</t>
+          <t>nodp-sweep.log</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -3763,19 +3763,19 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.005707</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>recorddp_pair_s42.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -3785,49 +3785,49 @@
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D110" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>0.000301</v>
+        <v>0.001897</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>recorddp_smoke.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D111" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.001957</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="112" ht="18" customHeight="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>recorddp_swap_s42.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -3841,19 +3841,19 @@
         </is>
       </c>
       <c r="D112" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.000237</v>
+        <v>0.005368</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>ref_e1000_group.log</t>
+          <t>rdp_e1000_s5.log</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -3870,7 +3870,7 @@
         <v>3</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>2.6e-05</v>
+        <v>0.004526</v>
       </c>
       <c r="F113" s="3" t="n">
         <v>1924</v>
@@ -3879,64 +3879,64 @@
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>rdp_eps_sweep.log</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.211667</v>
+        <v>0.003026</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>25143</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>recorddp_fast_s42.log</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.223153</v>
+        <v>0.288884</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>26892</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>recorddp_pair_s42.log</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -3945,76 +3945,76 @@
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.303531</v>
+        <v>0.000301</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>recorddp_smoke.log</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D117" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.378351</v>
+        <v>0.288884</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>25143</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>recorddp_swap_s42.log</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.428026</v>
+        <v>0.000237</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>26892</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>ref_e1000_group.log</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4026,16 +4026,16 @@
         <v>3</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>0.395166</v>
+        <v>2.6e-05</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -4061,7 +4061,7 @@
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -4087,7 +4087,7 @@
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -4113,7 +4113,7 @@
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -4127,19 +4127,19 @@
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>0.368463</v>
+        <v>0.378351</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -4153,19 +4153,19 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>0.378646</v>
+        <v>0.428026</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -4179,24 +4179,24 @@
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.373247</v>
+        <v>0.395166</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -4208,21 +4208,21 @@
         <v>10</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.211667</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -4234,21 +4234,21 @@
         <v>10</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.223153</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -4260,21 +4260,21 @@
         <v>10</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.303531</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -4286,7 +4286,7 @@
         <v>10</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.368463</v>
       </c>
       <c r="F129" s="3" t="n">
         <v>25200</v>
@@ -4295,12 +4295,12 @@
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -4312,7 +4312,7 @@
         <v>10</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.378646</v>
       </c>
       <c r="F130" s="3" t="n">
         <v>26829</v>
@@ -4321,12 +4321,12 @@
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -4338,7 +4338,7 @@
         <v>10</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.373247</v>
       </c>
       <c r="F131" s="3" t="n">
         <v>1341</v>
@@ -4347,12 +4347,12 @@
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -4364,7 +4364,7 @@
         <v>10</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.367252</v>
       </c>
       <c r="F132" s="3" t="n">
         <v>25200</v>
@@ -4373,12 +4373,12 @@
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -4390,7 +4390,7 @@
         <v>10</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.377587</v>
       </c>
       <c r="F133" s="3" t="n">
         <v>26829</v>
@@ -4399,12 +4399,12 @@
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -4416,7 +4416,7 @@
         <v>10</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.369278</v>
       </c>
       <c r="F134" s="3" t="n">
         <v>1341</v>
@@ -4425,12 +4425,12 @@
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -4439,10 +4439,10 @@
         </is>
       </c>
       <c r="D135" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F135" s="3" t="n">
         <v>25200</v>
@@ -4451,12 +4451,12 @@
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -4465,10 +4465,10 @@
         </is>
       </c>
       <c r="D136" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F136" s="3" t="n">
         <v>26829</v>
@@ -4477,12 +4477,12 @@
     <row r="137" ht="18" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4491,10 +4491,10 @@
         </is>
       </c>
       <c r="D137" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F137" s="3" t="n">
         <v>1341</v>
@@ -4503,7 +4503,7 @@
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -4517,10 +4517,10 @@
         </is>
       </c>
       <c r="D138" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F138" s="3" t="n">
         <v>25200</v>
@@ -4529,7 +4529,7 @@
     <row r="139" ht="18" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -4543,10 +4543,10 @@
         </is>
       </c>
       <c r="D139" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F139" s="3" t="n">
         <v>26829</v>
@@ -4555,7 +4555,7 @@
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -4569,10 +4569,10 @@
         </is>
       </c>
       <c r="D140" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F140" s="3" t="n">
         <v>1341</v>
@@ -4581,12 +4581,12 @@
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -4598,7 +4598,7 @@
         <v>3</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F141" s="3" t="n">
         <v>25200</v>
@@ -4607,12 +4607,12 @@
     <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -4624,7 +4624,7 @@
         <v>3</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F142" s="3" t="n">
         <v>26829</v>
@@ -4633,12 +4633,12 @@
     <row r="143" ht="18" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -4650,7 +4650,7 @@
         <v>3</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F143" s="3" t="n">
         <v>1341</v>
@@ -4659,7 +4659,7 @@
     <row r="144" ht="18" customHeight="1">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -4685,7 +4685,7 @@
     <row r="145" ht="18" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
     <row r="146" ht="18" customHeight="1">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4737,12 +4737,12 @@
     <row r="147" ht="18" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
@@ -4754,7 +4754,7 @@
         <v>3</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F147" s="3" t="n">
         <v>25200</v>
@@ -4763,12 +4763,12 @@
     <row r="148" ht="18" customHeight="1">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -4780,7 +4780,7 @@
         <v>3</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F148" s="3" t="n">
         <v>26829</v>
@@ -4789,26 +4789,182 @@
     <row r="149" ht="18" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F149" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F150" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F151" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="152" ht="18" customHeight="1">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
           <t>verify-sigma-fix.log</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
-        <is>
-          <t>no-DP</t>
-        </is>
-      </c>
-      <c r="C149" s="3" t="inlineStr">
-        <is>
-          <t>office1</t>
-        </is>
-      </c>
-      <c r="D149" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E149" s="3" t="n">
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E153" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F153" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="154" ht="18" customHeight="1">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F154" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E155" s="3" t="n">
         <v>0.006995</v>
       </c>
-      <c r="F149" s="3" t="n">
+      <c r="F155" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -4928,50 +5084,50 @@
     <row r="2" ht="80" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>central eps=1.0</t>
+          <t>central, eps=0.1</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.385978</v>
+        <v>0.435625</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>158.3</v>
+        <v>274.9</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.291187</v>
+        <v>0.481279</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>108.1</v>
+        <v>287.1</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.4997</v>
+        <v>0.5</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.4992</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.5063</v>
+        <v>0.5004999999999999</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.5027</v>
+        <v>0.502</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.0103</v>
+        <v>0.0105</v>
       </c>
       <c r="L2" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M2" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="N2" s="3" t="n">
-        <v>0.999909</v>
+        <v>0.462117</v>
       </c>
       <c r="O2" s="3" t="n">
-        <v>0.999955</v>
+        <v>0.731059</v>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
@@ -4982,38 +5138,38 @@
     <row r="3" ht="80" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>central eps=0.5</t>
+          <t>central, eps=0.5</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.454904</v>
+        <v>0.44151</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>186.6</v>
+        <v>278.6</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.474589</v>
+        <v>0.476242</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>176.2</v>
+        <v>284.1</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>0.4991</v>
+        <v>0.5002</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.4987</v>
+        <v>0.4996</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.5002</v>
+        <v>0.4999</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.5016</v>
+        <v>0.5003</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="L3" s="3" t="n">
         <v>0.5</v>
@@ -5036,50 +5192,50 @@
     <row r="4" ht="80" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>central eps=0.1</t>
+          <t>central, eps=1.0</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.435625</v>
+        <v>0.4144</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>178.7</v>
+        <v>261.5</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.481279</v>
+        <v>0.399209</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>178.7</v>
+        <v>238.1</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.5006</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.4992</v>
+        <v>0.5001</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0.5004999999999999</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.502</v>
+        <v>0.5024</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.0105</v>
+        <v>0.0102</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.462117</v>
+        <v>0.999909</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.731059</v>
+        <v>0.999955</v>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
@@ -5090,104 +5246,104 @@
     <row r="5" ht="80" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=16.0</t>
+          <t>dp-fedavg, eps=0.1</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.115064</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>47.2</v>
+        <v>0.422825</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>266.8</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.006265</v>
+        <v>0.422351</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2.3</v>
+        <v>251.9</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.5011</v>
+        <v>0.4995</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.5008</v>
+        <v>0.4994</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.4999</v>
+        <v>0.4997</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4996</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0.0097</v>
+        <v>0.0089</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>16</v>
+        <v>0.1</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>160</v>
+        <v>1</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>1</v>
+        <v>0.462117</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1</v>
+        <v>0.731059</v>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>COSTO OLTRE LA SOGLIA DI 3x (sezione 0 di ESPERIMENTI.md). bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=8.0</t>
+          <t>dp-fedavg, eps=0.5</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.225233</v>
+        <v>0.407656</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>92.40000000000001</v>
+        <v>257.2</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.056644</v>
+        <v>0.422867</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>21</v>
+        <v>252.2</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0.4998</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.5001</v>
+        <v>0.4993</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.4993</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.4979</v>
+        <v>0.498</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.0095</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>8</v>
+        <v>0.5</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>1</v>
+        <v>0.986614</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>1</v>
+        <v>0.9933070000000001</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
@@ -5198,50 +5354,50 @@
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=4.0</t>
+          <t>dp-fedavg, eps=1.0</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.298684</v>
+        <v>0.39476</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>122.5</v>
+        <v>249.1</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.127821</v>
+        <v>0.404192</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>47.5</v>
+        <v>241.1</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.4999</v>
+        <v>0.5002</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.5002</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.4988</v>
+        <v>0.4992</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.4959</v>
+        <v>0.4971</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>1</v>
+        <v>0.999909</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>1</v>
+        <v>0.999955</v>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
@@ -5252,44 +5408,44 @@
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=2.0</t>
+          <t>dp-fedavg, eps=16.0</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.365534</v>
+        <v>0.09454799999999999</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>149.9</v>
+        <v>59.7</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.274026</v>
+        <v>0.00614</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>101.7</v>
+        <v>3.7</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.5004</v>
+        <v>0.5014999999999999</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.5004999999999999</v>
+        <v>0.5011</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.4989</v>
+        <v>0.4997</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.4957</v>
+        <v>0.4992</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0097</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>20</v>
+        <v>160</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>1</v>
@@ -5306,50 +5462,50 @@
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=1.0</t>
+          <t>dp-fedavg, eps=2.0</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.39186</v>
+        <v>0.365534</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>160.7</v>
+        <v>230.6</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.344612</v>
+        <v>0.284881</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>127.9</v>
+        <v>169.9</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.5004</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.4996</v>
+        <v>0.5004999999999999</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.4991</v>
+        <v>0.4989</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.4975</v>
+        <v>0.4957</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0.0104</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="L9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N9" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M9" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="N9" s="3" t="n">
-        <v>0.999909</v>
-      </c>
       <c r="O9" s="3" t="n">
-        <v>0.999955</v>
+        <v>1</v>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
@@ -5360,50 +5516,50 @@
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=0.5</t>
+          <t>dp-fedavg, eps=4.0</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.407656</v>
+        <v>0.298684</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>167.2</v>
+        <v>188.4</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.422867</v>
+        <v>0.127821</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>157</v>
+        <v>76.2</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4999</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.5002</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.4988</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.4978</v>
+        <v>0.4959</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.0098</v>
+        <v>0.0092</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.986614</v>
+        <v>1</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>0.9933070000000001</v>
+        <v>1</v>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
@@ -5414,50 +5570,50 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg eps=0.1</t>
+          <t>dp-fedavg, eps=8.0</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.422825</v>
+        <v>0.190079</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>173.4</v>
+        <v>119.9</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.422351</v>
+        <v>0.065473</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>156.8</v>
+        <v>39.1</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.5001</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.5002</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4997</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.4991</v>
+        <v>0.4978</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0101</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="M11" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="N11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N11" s="3" t="n">
-        <v>0.462117</v>
-      </c>
       <c r="O11" s="3" t="n">
-        <v>0.731059</v>
+        <v>1</v>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
@@ -5468,50 +5624,50 @@
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>local eps=1.0</t>
+          <t>local, eps=0.1</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.384188</v>
+        <v>0.422825</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>157.6</v>
+        <v>266.8</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.375652</v>
+        <v>0.422351</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>139.5</v>
+        <v>251.9</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.4996</v>
+        <v>0.4995</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.4994</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.4992</v>
+        <v>0.4999</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.4984</v>
+        <v>0.4986</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0108</v>
+        <v>0.0092</v>
       </c>
       <c r="L12" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="M12" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="N12" s="3" t="n">
-        <v>0.999909</v>
+        <v>0.462117</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.999955</v>
+        <v>0.731059</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
@@ -5522,38 +5678,38 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>local eps=0.5</t>
+          <t>local, eps=0.5</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.397979</v>
+        <v>0.407656</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>163.3</v>
+        <v>257.2</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.411787</v>
+        <v>0.422867</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>152.9</v>
+        <v>252.2</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>0.4998</v>
       </c>
       <c r="H13" s="3" t="n">
+        <v>0.4993</v>
+      </c>
+      <c r="I13" s="3" t="n">
         <v>0.4995</v>
       </c>
-      <c r="I13" s="3" t="n">
-        <v>0.4997</v>
-      </c>
       <c r="J13" s="3" t="n">
-        <v>0.4978</v>
+        <v>0.4975</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0.0106</v>
+        <v>0.0101</v>
       </c>
       <c r="L13" s="3" t="n">
         <v>0.5</v>
@@ -5576,50 +5732,50 @@
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>local eps=0.1</t>
+          <t>local, eps=1.0</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.422283</v>
+        <v>0.39476</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>173.2</v>
+        <v>249.1</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.419873</v>
+        <v>0.404192</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>155.9</v>
+        <v>241.1</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.5002</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.4992</v>
+        <v>0.5</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.5</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.4987</v>
+        <v>0.4983</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0108</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.462117</v>
+        <v>0.999909</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.731059</v>
+        <v>0.999955</v>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -5630,38 +5786,38 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>no-DP baseline</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.002438</v>
+        <v>0.001585</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.002693</v>
+        <v>0.001677</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.5027</v>
+        <v>0.5003</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.5011</v>
+        <v>0.5016</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0.5096000000000001</v>
+        <v>0.5003</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.5129</v>
+        <v>0.5004</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0.0098</v>
+        <v>0.0105</v>
       </c>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>

</xml_diff>

<commit_message>
RQ2: E-D senza DP analizzato (foglio RQ2_partizione, seg 45, 55); punto operativo C=1 eps=64; config di E-D con DP; SprintLog 10zz+129/130
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costo_per_sito" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utility_privacy_limite" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worst_case_per_record" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossario_metriche" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RQ2_partizione" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossario_metriche" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrice_sintesi'!$A$1:$I$1</definedName>
@@ -561,7 +562,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>158 run in regime naturale</t>
+          <t>160 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -613,7 +614,7 @@
     <row r="3" ht="160" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>260 run totali</t>
+          <t>10 run E-D senza DP (seconda macchina)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -621,9 +622,9 @@
           <t>RQ2</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>lacuna strutturale</t>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>completata da verificare</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -633,17 +634,17 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si, appaiando per seed</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Non esiste alcun riferimento IID. I client sono i 3 siti reali, quindi l'eterogeneita' non e' un fattore manipolato ma una proprieta' dei dati. Nessuna run puo' colmarla a posteriori.</t>
+          <t>Braccio senza DP eseguito. Loss sull'holdout del modello rilasciato, IID contro per sito: 0.001330 contro 0.001615 (t = -1.26, 4 gdl); Yeom 0.5011 contro 0.5001. Manca il braccio con DP.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Costruire la partizione IID rimescolando le sessioni fra i siti a parita' di numerosita' per client, poi IID/non-IID x senza-DP/con-DP: 4 celle x 5 seed = 20 run.</t>
+          <t>IID e per sito al punto operativo client-level: 2 celle x 5 seed = 10 run; la cella per sito coincide con quella di RQ1 al punto operativo.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -653,19 +654,19 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>La guida (Fase E) avverte che una partizione IID artificiale e' un riferimento sperimentale, non un deployment reale: va dichiarato.</t>
+          <t>Partizione IID = riferimento sperimentale, non un deployment: va dichiarato. Macchina diversa da E-A: variabile da dichiarare.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Fase A -&gt; E</t>
+          <t>Fase E</t>
         </is>
       </c>
     </row>
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>260 run totali</t>
+          <t>262 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -921,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F155"/>
+  <dimension ref="A1:F164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3775,12 +3776,12 @@
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.25_eps16.log</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -3792,7 +3793,7 @@
         <v>10</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>0.001897</v>
+        <v>0.004529</v>
       </c>
       <c r="F110" s="3" t="n">
         <v>25200</v>
@@ -3801,12 +3802,12 @@
     <row r="111" ht="18" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.25_eps16.log</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -3818,7 +3819,7 @@
         <v>10</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>0.001957</v>
+        <v>0.003908</v>
       </c>
       <c r="F111" s="3" t="n">
         <v>26829</v>
@@ -3827,12 +3828,12 @@
     <row r="112" ht="18" customHeight="1">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.25_eps16.log</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -3844,7 +3845,7 @@
         <v>10</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0.005368</v>
+        <v>0.008791</v>
       </c>
       <c r="F112" s="3" t="n">
         <v>1341</v>
@@ -3853,64 +3854,64 @@
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>rdp_e1000_s5.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>0.004526</v>
+        <v>0.001159</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>rdp_eps_sweep.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.003026</v>
+        <v>0.000859</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>recorddp_fast_s42.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -3919,76 +3920,76 @@
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.008803</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>recorddp_pair_s42.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D116" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.000301</v>
+        <v>0.002695</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>recorddp_smoke.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D117" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.002637</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>recorddp_swap_s42.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -3997,19 +3998,19 @@
         </is>
       </c>
       <c r="D118" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.000237</v>
+        <v>0.006224</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>ref_e1000_group.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -4019,80 +4020,80 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D119" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>2.6e-05</v>
+        <v>0.001897</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D120" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>0.211667</v>
+        <v>0.001957</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>25143</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D121" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>0.223153</v>
+        <v>0.005368</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>26892</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>rdp_e1000_s5.log</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -4101,76 +4102,76 @@
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>0.303531</v>
+        <v>0.004526</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>rdp_eps_sweep.log</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D123" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>0.378351</v>
+        <v>0.003026</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>25143</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>recorddp_fast_s42.log</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>0.428026</v>
+        <v>0.288884</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>26892</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>recorddp_pair_s42.log</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -4182,73 +4183,73 @@
         <v>3</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.395166</v>
+        <v>0.000301</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>recorddp_smoke.log</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.211667</v>
+        <v>0.288884</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>25143</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>recorddp_swap_s42.log</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>0.223153</v>
+        <v>0.000237</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>26892</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>ref_e1000_group.log</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -4257,19 +4258,19 @@
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>0.303531</v>
+        <v>2.6e-05</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -4286,16 +4287,16 @@
         <v>10</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.368463</v>
+        <v>0.211667</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -4312,16 +4313,16 @@
         <v>10</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>0.378646</v>
+        <v>0.223153</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -4338,21 +4339,21 @@
         <v>10</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.373247</v>
+        <v>0.303531</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -4361,24 +4362,24 @@
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.378351</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -4387,24 +4388,24 @@
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.428026</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -4413,24 +4414,24 @@
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.395166</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -4442,21 +4443,21 @@
         <v>10</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.211667</v>
       </c>
       <c r="F135" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -4468,21 +4469,21 @@
         <v>10</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.223153</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="137" ht="18" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4494,21 +4495,21 @@
         <v>10</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.303531</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -4520,7 +4521,7 @@
         <v>10</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.368463</v>
       </c>
       <c r="F138" s="3" t="n">
         <v>25200</v>
@@ -4529,12 +4530,12 @@
     <row r="139" ht="18" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -4546,7 +4547,7 @@
         <v>10</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.378646</v>
       </c>
       <c r="F139" s="3" t="n">
         <v>26829</v>
@@ -4555,12 +4556,12 @@
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -4572,7 +4573,7 @@
         <v>10</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.373247</v>
       </c>
       <c r="F140" s="3" t="n">
         <v>1341</v>
@@ -4581,12 +4582,12 @@
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -4595,10 +4596,10 @@
         </is>
       </c>
       <c r="D141" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.367252</v>
       </c>
       <c r="F141" s="3" t="n">
         <v>25200</v>
@@ -4607,12 +4608,12 @@
     <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -4621,10 +4622,10 @@
         </is>
       </c>
       <c r="D142" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.377587</v>
       </c>
       <c r="F142" s="3" t="n">
         <v>26829</v>
@@ -4633,12 +4634,12 @@
     <row r="143" ht="18" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -4647,10 +4648,10 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.369278</v>
       </c>
       <c r="F143" s="3" t="n">
         <v>1341</v>
@@ -4659,12 +4660,12 @@
     <row r="144" ht="18" customHeight="1">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -4673,10 +4674,10 @@
         </is>
       </c>
       <c r="D144" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F144" s="3" t="n">
         <v>25200</v>
@@ -4685,12 +4686,12 @@
     <row r="145" ht="18" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -4699,10 +4700,10 @@
         </is>
       </c>
       <c r="D145" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F145" s="3" t="n">
         <v>26829</v>
@@ -4711,12 +4712,12 @@
     <row r="146" ht="18" customHeight="1">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -4725,10 +4726,10 @@
         </is>
       </c>
       <c r="D146" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F146" s="3" t="n">
         <v>1341</v>
@@ -4737,12 +4738,12 @@
     <row r="147" ht="18" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
@@ -4751,10 +4752,10 @@
         </is>
       </c>
       <c r="D147" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.002174</v>
       </c>
       <c r="F147" s="3" t="n">
         <v>25200</v>
@@ -4763,12 +4764,12 @@
     <row r="148" ht="18" customHeight="1">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -4777,10 +4778,10 @@
         </is>
       </c>
       <c r="D148" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002005</v>
       </c>
       <c r="F148" s="3" t="n">
         <v>26829</v>
@@ -4789,12 +4790,12 @@
     <row r="149" ht="18" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -4803,10 +4804,10 @@
         </is>
       </c>
       <c r="D149" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.005707</v>
       </c>
       <c r="F149" s="3" t="n">
         <v>1341</v>
@@ -4815,7 +4816,7 @@
     <row r="150" ht="18" customHeight="1">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -4841,7 +4842,7 @@
     <row r="151" ht="18" customHeight="1">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -4867,7 +4868,7 @@
     <row r="152" ht="18" customHeight="1">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -4893,7 +4894,7 @@
     <row r="153" ht="18" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
@@ -4919,7 +4920,7 @@
     <row r="154" ht="18" customHeight="1">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
@@ -4945,7 +4946,7 @@
     <row r="155" ht="18" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -4965,6 +4966,240 @@
         <v>0.006995</v>
       </c>
       <c r="F155" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>0.086894</v>
+      </c>
+      <c r="F156" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E157" s="3" t="n">
+        <v>0.076844</v>
+      </c>
+      <c r="F157" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F158" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E159" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F159" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F160" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="161" ht="18" customHeight="1">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E161" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F161" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="162" ht="18" customHeight="1">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F162" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E163" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F163" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="164" ht="18" customHeight="1">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E164" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F164" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -5840,7 +6075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6345,8 +6580,110 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="10" ht="76" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>rq2-per_site</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>289.99</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>8.827</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>7.156</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>1.231</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>-0.329</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.2203</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>-1.494</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>1.651</v>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="76" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>rq2-iid</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>366</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>291.69</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>17.61</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>13.481</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>-5.833</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0.2215</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>-0.153</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>2.084</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>1.661</v>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>
@@ -6358,6 +6695,883 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>per sito, media (5 seed)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>IID, media</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>differenza appaiata IID - per sito</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>deviazione standard</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>t (4 gdl)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>seed con IID sotto per sito</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>nodp-sweep2, media (prima macchina, stesso config di per sito)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>lettura</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.001615</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.00133</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>-0.000286</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.000509</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>-1.26</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.001585</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.001337</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.001055</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>-0.000282</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.00048</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.00131</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.000278</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.000274</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>-4e-06</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>7.9e-05</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2 su 5</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.000275</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.001712</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.001495</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>-0.000217</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.00047</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.001677</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.500089</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.501123</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.001034</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.004061</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2 su 5</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.50018</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.500367</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.501129</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.000762</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.002938</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>1 su 5</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0.500262</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.501362</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.501232</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>-0.00013</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.001538</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0.501601</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.498234</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.499349</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.001115</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.004366</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2 su 5</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.500367</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.009101</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.008920000000000001</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>-0.000181</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.001959</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0.01048</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>il caso vale 0.01; nessuna differenza significativa</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>braccio</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.001854</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.001627</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.000227</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0.001973</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0.497489</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0.496833</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.497304</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0.49799</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0.01057</v>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.001543</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.001212</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.000331</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.001627</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.5004150000000001</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.498608</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.498715</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.501325</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.009519</v>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.002015</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.001585</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.00043</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.001997</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.498318</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.499253</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.501857</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.496275</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0.008544</v>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.001251</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.000937</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.000314</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.001395</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.500512</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.499806</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.501676</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.493375</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0.008695</v>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.000717</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.000646</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>7.1e-05</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0.0009840000000000001</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0.500217</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.501356</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.502413</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0.494383</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0.007123</v>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.001287</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.001204</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>8.3e-05</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.001585</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.506096</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.506139</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.503836</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.500351</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.010194</v>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.001586</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.001316</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.00027</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0.001711</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.503578</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.503702</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.502437</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0.5002490000000001</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0.008397</v>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.001201</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.000923</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.000278</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.001392</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.498879</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.500372</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.500932</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0.496163</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0.007197</v>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>0.001904</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.001511</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0.000393</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0.001894</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0.500845</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0.500694</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0.5028</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0.502273</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0.01087</v>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.001367</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.001001</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.000366</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.001478</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.499713</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.5007200000000001</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.501004</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.505533</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0.008996000000000001</v>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="3" t="n"/>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Fonte: experiments_altre_macchine/rq2-per_site e rq2-iid (E-D, senza DP, seconda macchina, commit 3815da7). I due bracci differiscono solo per partition.strategy e sono appaiati per seed. La partizione IID rimescola le sessioni fra i siti conservando le numerosita' per client: e' un riferimento sperimentale, non un deployment. nodp-sweep2 e' la stessa configurazione del braccio per sito su un'altra macchina e un altro commit: la loss sull'holdout differisce per seed fino al 23% (segnalazione 45), per questo il confronto di RQ2 non la usa.</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
RQ1: griglia del punto operativo completa, punto C=1 eps=64; config eps=32; seg 55 confermata; SprintLog 10zz+132
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -562,7 +562,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>160 run in regime naturale</t>
+          <t>166 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>262 run totali</t>
+          <t>268 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -922,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3854,12 +3854,12 @@
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>op_C0.25_eps64.log</t>
+          <t>op_C0.25_eps256.log</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=64.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -3868,10 +3868,10 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>0.001159</v>
+        <v>0.005606</v>
       </c>
       <c r="F113" s="3" t="n">
         <v>25200</v>
@@ -3880,12 +3880,12 @@
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>op_C0.25_eps64.log</t>
+          <t>op_C0.25_eps256.log</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=64.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -3894,10 +3894,10 @@
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0.000859</v>
+        <v>0.004914</v>
       </c>
       <c r="F114" s="3" t="n">
         <v>26829</v>
@@ -3906,12 +3906,12 @@
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>op_C0.25_eps64.log</t>
+          <t>op_C0.25_eps256.log</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=64.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -3920,10 +3920,10 @@
         </is>
       </c>
       <c r="D115" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0.008803</v>
+        <v>0.009353</v>
       </c>
       <c r="F115" s="3" t="n">
         <v>1341</v>
@@ -3932,7 +3932,7 @@
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>op_eps64.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3949,7 +3949,7 @@
         <v>10</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0.002695</v>
+        <v>0.004537</v>
       </c>
       <c r="F116" s="3" t="n">
         <v>25200</v>
@@ -3958,7 +3958,7 @@
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>op_eps64.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -3975,7 +3975,7 @@
         <v>10</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>0.002637</v>
+        <v>0.004089</v>
       </c>
       <c r="F117" s="3" t="n">
         <v>26829</v>
@@ -3984,7 +3984,7 @@
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>op_eps64.log</t>
+          <t>op_C0.25_eps64.log</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -4001,7 +4001,7 @@
         <v>10</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>0.006224</v>
+        <v>0.008904</v>
       </c>
       <c r="F118" s="3" t="n">
         <v>1341</v>
@@ -4010,12 +4010,12 @@
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.5_eps16.log</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4027,7 +4027,7 @@
         <v>10</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>0.001897</v>
+        <v>0.003457</v>
       </c>
       <c r="F119" s="3" t="n">
         <v>25200</v>
@@ -4036,12 +4036,12 @@
     <row r="120" ht="18" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.5_eps16.log</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -4053,7 +4053,7 @@
         <v>10</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>0.001957</v>
+        <v>0.003445</v>
       </c>
       <c r="F120" s="3" t="n">
         <v>26829</v>
@@ -4062,12 +4062,12 @@
     <row r="121" ht="18" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>prova_recorddp_s42_attacchi_saltati.log</t>
+          <t>op_C0.5_eps16.log</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=16.0)</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -4079,7 +4079,7 @@
         <v>10</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>0.005368</v>
+        <v>0.006348</v>
       </c>
       <c r="F121" s="3" t="n">
         <v>1341</v>
@@ -4088,64 +4088,64 @@
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>rdp_e1000_s5.log</t>
+          <t>op_C0.5_eps256.log</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D122" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>0.004526</v>
+        <v>0.003837</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>rdp_eps_sweep.log</t>
+          <t>op_C0.5_eps256.log</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D123" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>0.003026</v>
+        <v>0.00347</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="124" ht="18" customHeight="1">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>recorddp_fast_s42.log</t>
+          <t>op_C0.5_eps256.log</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -4154,76 +4154,76 @@
         </is>
       </c>
       <c r="D124" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.007703</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="125" ht="18" customHeight="1">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>recorddp_pair_s42.log</t>
+          <t>op_C0.5_eps64.log</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D125" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>0.000301</v>
+        <v>0.002505</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>recorddp_smoke.log</t>
+          <t>op_C0.5_eps64.log</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D126" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>0.288884</v>
+        <v>0.002495</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>1924</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>recorddp_swap_s42.log</t>
+          <t>op_C0.5_eps64.log</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -4232,258 +4232,258 @@
         </is>
       </c>
       <c r="D127" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>0.000237</v>
+        <v>0.006796</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>1924</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>ref_e1000_group.log</t>
+          <t>op_eps256.log</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D128" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>2.6e-05</v>
+        <v>0.00226</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>1924</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>op_eps256.log</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D129" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>0.211667</v>
+        <v>0.00237</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>25143</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>op_eps256.log</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=256.0)</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D130" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>0.223153</v>
+        <v>0.006203</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>26892</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="131" ht="18" customHeight="1">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D131" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>0.303531</v>
+        <v>0.002695</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>1335</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="132" ht="18" customHeight="1">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D132" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>0.378351</v>
+        <v>0.002637</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>25143</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>op_eps64.log</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D133" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0.428026</v>
+        <v>0.006224</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>26892</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="134" ht="18" customHeight="1">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>office1</t>
+          <t>caltech</t>
         </is>
       </c>
       <c r="D134" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>0.395166</v>
+        <v>0.001897</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>1335</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="135" ht="18" customHeight="1">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>jpl</t>
         </is>
       </c>
       <c r="D135" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>0.211667</v>
+        <v>0.001957</v>
       </c>
       <c r="F135" s="3" t="n">
-        <v>25143</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="136" ht="18" customHeight="1">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>prova_recorddp_s42_attacchi_saltati.log</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D136" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>0.223153</v>
+        <v>0.005368</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>26892</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="137" ht="18" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
+          <t>rdp_e1000_s5.log</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -4492,76 +4492,76 @@
         </is>
       </c>
       <c r="D137" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>0.303531</v>
+        <v>0.004526</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>1335</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="138" ht="18" customHeight="1">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rdp_eps_sweep.log</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D138" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>0.368463</v>
+        <v>0.003026</v>
       </c>
       <c r="F138" s="3" t="n">
-        <v>25200</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="139" ht="18" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>recorddp_fast_s42.log</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D139" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>0.378646</v>
+        <v>0.288884</v>
       </c>
       <c r="F139" s="3" t="n">
-        <v>26829</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>recorddp_pair_s42.log</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -4570,76 +4570,76 @@
         </is>
       </c>
       <c r="D140" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>0.373247</v>
+        <v>0.000301</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>1341</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>recorddp_smoke.log</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>caltech</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D141" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.288884</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>25200</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="142" ht="18" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>recorddp_swap_s42.log</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>jpl</t>
+          <t>office1</t>
         </is>
       </c>
       <c r="D142" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.000237</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>26829</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="143" ht="18" customHeight="1">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>ref_e1000_group.log</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -4648,24 +4648,24 @@
         </is>
       </c>
       <c r="D143" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>0.369278</v>
+        <v>2.6e-05</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>1341</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="144" ht="18" customHeight="1">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -4677,21 +4677,21 @@
         <v>10</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.211667</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="145" ht="18" customHeight="1">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -4703,21 +4703,21 @@
         <v>10</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.223153</v>
       </c>
       <c r="F145" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="146" ht="18" customHeight="1">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq1_eps2_seed789_rerun.log</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -4729,21 +4729,21 @@
         <v>10</v>
       </c>
       <c r="E146" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.303531</v>
       </c>
       <c r="F146" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="147" ht="18" customHeight="1">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
@@ -4752,24 +4752,24 @@
         </is>
       </c>
       <c r="D147" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.378351</v>
       </c>
       <c r="F147" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="148" ht="18" customHeight="1">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -4778,24 +4778,24 @@
         </is>
       </c>
       <c r="D148" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E148" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.428026</v>
       </c>
       <c r="F148" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="149" ht="18" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>rq1_eps2_seed789_rerun3_annullato.log</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -4804,24 +4804,24 @@
         </is>
       </c>
       <c r="D149" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.395166</v>
       </c>
       <c r="F149" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="150" ht="18" customHeight="1">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
@@ -4830,24 +4830,24 @@
         </is>
       </c>
       <c r="D150" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E150" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.211667</v>
       </c>
       <c r="F150" s="3" t="n">
-        <v>25200</v>
+        <v>25143</v>
       </c>
     </row>
     <row r="151" ht="18" customHeight="1">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
@@ -4856,24 +4856,24 @@
         </is>
       </c>
       <c r="D151" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223153</v>
       </c>
       <c r="F151" s="3" t="n">
-        <v>26829</v>
+        <v>26892</v>
       </c>
     </row>
     <row r="152" ht="18" customHeight="1">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>rq1_eps2_seed789_rerun_interrotto.log</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
@@ -4882,24 +4882,24 @@
         </is>
       </c>
       <c r="D152" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E152" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.303531</v>
       </c>
       <c r="F152" s="3" t="n">
-        <v>1341</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="153" ht="18" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
@@ -4908,10 +4908,10 @@
         </is>
       </c>
       <c r="D153" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.368463</v>
       </c>
       <c r="F153" s="3" t="n">
         <v>25200</v>
@@ -4920,12 +4920,12 @@
     <row r="154" ht="18" customHeight="1">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -4934,10 +4934,10 @@
         </is>
       </c>
       <c r="D154" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E154" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.378646</v>
       </c>
       <c r="F154" s="3" t="n">
         <v>26829</v>
@@ -4946,12 +4946,12 @@
     <row r="155" ht="18" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
@@ -4960,10 +4960,10 @@
         </is>
       </c>
       <c r="D155" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E155" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.373247</v>
       </c>
       <c r="F155" s="3" t="n">
         <v>1341</v>
@@ -4972,12 +4972,12 @@
     <row r="156" ht="18" customHeight="1">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
@@ -4986,10 +4986,10 @@
         </is>
       </c>
       <c r="D156" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.367252</v>
       </c>
       <c r="F156" s="3" t="n">
         <v>25200</v>
@@ -4998,12 +4998,12 @@
     <row r="157" ht="18" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
@@ -5012,10 +5012,10 @@
         </is>
       </c>
       <c r="D157" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.377587</v>
       </c>
       <c r="F157" s="3" t="n">
         <v>26829</v>
@@ -5024,12 +5024,12 @@
     <row r="158" ht="18" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -5038,10 +5038,10 @@
         </is>
       </c>
       <c r="D158" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.369278</v>
       </c>
       <c r="F158" s="3" t="n">
         <v>1341</v>
@@ -5050,12 +5050,12 @@
     <row r="159" ht="18" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
@@ -5064,10 +5064,10 @@
         </is>
       </c>
       <c r="D159" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F159" s="3" t="n">
         <v>25200</v>
@@ -5076,12 +5076,12 @@
     <row r="160" ht="18" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -5090,10 +5090,10 @@
         </is>
       </c>
       <c r="D160" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F160" s="3" t="n">
         <v>26829</v>
@@ -5102,12 +5102,12 @@
     <row r="161" ht="18" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
@@ -5116,10 +5116,10 @@
         </is>
       </c>
       <c r="D161" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F161" s="3" t="n">
         <v>1341</v>
@@ -5128,7 +5128,7 @@
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -5142,10 +5142,10 @@
         </is>
       </c>
       <c r="D162" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F162" s="3" t="n">
         <v>25200</v>
@@ -5154,7 +5154,7 @@
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -5168,10 +5168,10 @@
         </is>
       </c>
       <c r="D163" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F163" s="3" t="n">
         <v>26829</v>
@@ -5180,26 +5180,416 @@
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
+          <t>verify-10rounds-nodp.log</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E164" s="3" t="n">
+        <v>0.005707</v>
+      </c>
+      <c r="F164" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="165" ht="18" customHeight="1">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>verify-mu-anchor.log</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E165" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F165" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>verify-mu-anchor.log</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E166" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F166" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>verify-mu-anchor.log</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E167" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F167" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>verify-outlier-fix.log</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F168" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>verify-outlier-fix.log</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E169" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F169" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>verify-outlier-fix.log</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E170" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F170" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E171" s="3" t="n">
+        <v>0.086894</v>
+      </c>
+      <c r="F171" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E172" s="3" t="n">
+        <v>0.076844</v>
+      </c>
+      <c r="F172" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="173" ht="18" customHeight="1">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-central.log</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>DP (eps=1.0)</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E173" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F173" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="174" ht="18" customHeight="1">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E174" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F174" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="175" ht="18" customHeight="1">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E175" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F175" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="176" ht="18" customHeight="1">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E176" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F176" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="177" ht="18" customHeight="1">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
           <t>verify-sigma-fix.log</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
-        <is>
-          <t>no-DP</t>
-        </is>
-      </c>
-      <c r="C164" s="3" t="inlineStr">
-        <is>
-          <t>office1</t>
-        </is>
-      </c>
-      <c r="D164" s="3" t="n">
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E164" s="3" t="n">
+      <c r="E177" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F177" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="178" ht="18" customHeight="1">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E178" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F178" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="179" ht="18" customHeight="1">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E179" s="3" t="n">
         <v>0.006995</v>
       </c>
-      <c r="F164" s="3" t="n">
+      <c r="F179" s="3" t="n">
         <v>1341</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RQ1: punto operativo a 5 seed, 4.5 volte il no-DP, nessuna configurazione client-level sotto 3; eps=32; test per record a eps=64; SprintLog 10zz+133
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -562,7 +562,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>166 run in regime naturale</t>
+          <t>172 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>268 run totali</t>
+          <t>274 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -922,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4894,12 +4894,12 @@
     <row r="153" ht="18" customHeight="1">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps64.log</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
@@ -4911,21 +4911,21 @@
         <v>10</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>0.368463</v>
+        <v>0.002448</v>
       </c>
       <c r="F153" s="3" t="n">
-        <v>25200</v>
+        <v>25239</v>
       </c>
     </row>
     <row r="154" ht="18" customHeight="1">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps64.log</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -4937,21 +4937,21 @@
         <v>10</v>
       </c>
       <c r="E154" s="3" t="n">
-        <v>0.378646</v>
+        <v>0.00288</v>
       </c>
       <c r="F154" s="3" t="n">
-        <v>26829</v>
+        <v>26781</v>
       </c>
     </row>
     <row r="155" ht="18" customHeight="1">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>rq1_eps_sweep.log</t>
+          <t>rq1_eps64.log</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=2.0)</t>
+          <t>DP (eps=64.0)</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
@@ -4963,21 +4963,21 @@
         <v>10</v>
       </c>
       <c r="E155" s="3" t="n">
-        <v>0.373247</v>
+        <v>0.005745</v>
       </c>
       <c r="F155" s="3" t="n">
-        <v>1341</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="156" ht="18" customHeight="1">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
@@ -4989,7 +4989,7 @@
         <v>10</v>
       </c>
       <c r="E156" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.368463</v>
       </c>
       <c r="F156" s="3" t="n">
         <v>25200</v>
@@ -4998,12 +4998,12 @@
     <row r="157" ht="18" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
@@ -5015,7 +5015,7 @@
         <v>10</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.378646</v>
       </c>
       <c r="F157" s="3" t="n">
         <v>26829</v>
@@ -5024,12 +5024,12 @@
     <row r="158" ht="18" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_eps_sweep.log</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>DP (eps=2.0)</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
         <v>10</v>
       </c>
       <c r="E158" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.373247</v>
       </c>
       <c r="F158" s="3" t="n">
         <v>1341</v>
@@ -5050,12 +5050,12 @@
     <row r="159" ht="18" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
@@ -5067,7 +5067,7 @@
         <v>10</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.367252</v>
       </c>
       <c r="F159" s="3" t="n">
         <v>25200</v>
@@ -5076,12 +5076,12 @@
     <row r="160" ht="18" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -5093,7 +5093,7 @@
         <v>10</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.377587</v>
       </c>
       <c r="F160" s="3" t="n">
         <v>26829</v>
@@ -5102,12 +5102,12 @@
     <row r="161" ht="18" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
@@ -5119,7 +5119,7 @@
         <v>10</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.369278</v>
       </c>
       <c r="F161" s="3" t="n">
         <v>1341</v>
@@ -5128,12 +5128,12 @@
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -5145,7 +5145,7 @@
         <v>10</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.195433</v>
       </c>
       <c r="F162" s="3" t="n">
         <v>25200</v>
@@ -5154,12 +5154,12 @@
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
@@ -5171,7 +5171,7 @@
         <v>10</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.223175</v>
       </c>
       <c r="F163" s="3" t="n">
         <v>26829</v>
@@ -5180,12 +5180,12 @@
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -5197,7 +5197,7 @@
         <v>10</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.353804</v>
       </c>
       <c r="F164" s="3" t="n">
         <v>1341</v>
@@ -5206,7 +5206,7 @@
     <row r="165" ht="18" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -5220,10 +5220,10 @@
         </is>
       </c>
       <c r="D165" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F165" s="3" t="n">
         <v>25200</v>
@@ -5232,7 +5232,7 @@
     <row r="166" ht="18" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -5246,10 +5246,10 @@
         </is>
       </c>
       <c r="D166" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F166" s="3" t="n">
         <v>26829</v>
@@ -5258,7 +5258,7 @@
     <row r="167" ht="18" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -5272,10 +5272,10 @@
         </is>
       </c>
       <c r="D167" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F167" s="3" t="n">
         <v>1341</v>
@@ -5284,7 +5284,7 @@
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -5310,7 +5310,7 @@
     <row r="169" ht="18" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -5336,7 +5336,7 @@
     <row r="170" ht="18" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -5362,12 +5362,12 @@
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
@@ -5379,7 +5379,7 @@
         <v>3</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F171" s="3" t="n">
         <v>25200</v>
@@ -5388,12 +5388,12 @@
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -5405,7 +5405,7 @@
         <v>3</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F172" s="3" t="n">
         <v>26829</v>
@@ -5414,12 +5414,12 @@
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
@@ -5431,7 +5431,7 @@
         <v>3</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F173" s="3" t="n">
         <v>1341</v>
@@ -5440,12 +5440,12 @@
     <row r="174" ht="18" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -5457,7 +5457,7 @@
         <v>3</v>
       </c>
       <c r="E174" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F174" s="3" t="n">
         <v>25200</v>
@@ -5466,12 +5466,12 @@
     <row r="175" ht="18" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
@@ -5483,7 +5483,7 @@
         <v>3</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F175" s="3" t="n">
         <v>26829</v>
@@ -5492,12 +5492,12 @@
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -5509,7 +5509,7 @@
         <v>3</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.120528</v>
       </c>
       <c r="F176" s="3" t="n">
         <v>1341</v>
@@ -5518,7 +5518,7 @@
     <row r="177" ht="18" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -5544,7 +5544,7 @@
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -5570,7 +5570,7 @@
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -5590,6 +5590,84 @@
         <v>0.006995</v>
       </c>
       <c r="F179" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="180" ht="18" customHeight="1">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E180" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F180" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="181" ht="18" customHeight="1">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E181" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F181" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="182" ht="18" customHeight="1">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E182" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F182" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -5604,7 +5682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6195,44 +6273,44 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>dp-fedavg, eps=8.0</t>
+          <t>dp-fedavg, eps=64.0</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.190079</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>119.9</v>
+        <v>0.007116</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>4.5</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.065473</v>
+        <v>0.002651</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>39.1</v>
+        <v>1.6</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.5001</v>
+        <v>0.5004</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.5002</v>
+        <v>0.5013</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.4997</v>
+        <v>0.4996</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.4978</v>
+        <v>0.5011</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.0105</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>80</v>
+        <v>640</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>1</v>
@@ -6242,57 +6320,57 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+          <t>COSTO OLTRE LA SOGLIA DI 3x (sezione 0 di ESPERIMENTI.md). bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
         </is>
       </c>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>local, eps=0.1</t>
+          <t>dp-fedavg, eps=8.0</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.422825</v>
+        <v>0.190079</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>266.8</v>
+        <v>119.9</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.422351</v>
+        <v>0.065473</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>251.9</v>
+        <v>39.1</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.5001</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.4994</v>
+        <v>0.5002</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.4999</v>
+        <v>0.4997</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.4986</v>
+        <v>0.4978</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.0101</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="M12" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="N12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N12" s="3" t="n">
-        <v>0.462117</v>
-      </c>
       <c r="O12" s="3" t="n">
-        <v>0.731059</v>
+        <v>1</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
@@ -6303,50 +6381,50 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>local, eps=0.5</t>
+          <t>local, eps=0.1</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.407656</v>
+        <v>0.422825</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>257.2</v>
+        <v>266.8</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.422867</v>
+        <v>0.422351</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>252.2</v>
+        <v>251.9</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.4998</v>
+        <v>0.4995</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.4993</v>
+        <v>0.4994</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.4999</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.4975</v>
+        <v>0.4986</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0.0101</v>
+        <v>0.0092</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.986614</v>
+        <v>0.462117</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>0.9933070000000001</v>
+        <v>0.731059</v>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
@@ -6357,50 +6435,50 @@
     <row r="14" ht="80" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>local, eps=1.0</t>
+          <t>local, eps=0.5</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.39476</v>
+        <v>0.407656</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>249.1</v>
+        <v>257.2</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.404192</v>
+        <v>0.422867</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>241.1</v>
+        <v>252.2</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.5002</v>
+        <v>0.4998</v>
       </c>
       <c r="H14" s="3" t="n">
+        <v>0.4993</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.4995</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.4975</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.0101</v>
+      </c>
+      <c r="L14" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="I14" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>0.4983</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>0.0108</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="M14" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>0.999909</v>
+        <v>0.986614</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>0.999955</v>
+        <v>0.9933070000000001</v>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
@@ -6411,44 +6489,98 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>no-DP baseline</t>
+          <t>local, eps=1.0</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="3" t="n">
+        <v>0.39476</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>249.1</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.404192</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>241.1</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.5002</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.4983</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>0.999909</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>0.999955</v>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>UTILITY DISTRUTTA (loss sull'holdout del modello rilasciato oltre 50x il riferimento): un nullo di privacy qui non distingue 'DP protegge' da 'il modello non impara, quindi non memorizza'. bound VACUO: a questo eps cumulativo la garanzia permette un attacco quasi perfetto, quindi 'siamo sotto il limite' non e' informativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>no-DP baseline</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="3" t="n">
         <v>0.001585</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D16" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E16" s="3" t="n">
         <v>0.001677</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F16" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G16" s="3" t="n">
         <v>0.5003</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H16" s="3" t="n">
         <v>0.5016</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I16" s="3" t="n">
         <v>0.5003</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J16" s="3" t="n">
         <v>0.5004</v>
       </c>
-      <c r="K15" s="3" t="n">
+      <c r="K16" s="3" t="n">
         <v>0.0105</v>
       </c>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="n"/>
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>riferimento senza DP: nessuna garanzia da confrontare</t>
         </is>
@@ -6465,7 +6597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7072,8 +7204,59 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="12" ht="76" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>dp-fedavg_eps64</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>473</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>290.31</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>15.74</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>11.607</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>10.354</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.734</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0.2201</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>2.693</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>1.653</v>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>

</xml_diff>

<commit_message>
RQ2: braccio con DP di E-D (eps=64, C=1), foglio RQ2_partizione completo, test per record dei bracci con DP; E-B seed 123; SprintLog 10zz+134
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -639,12 +639,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Braccio senza DP eseguito. Loss sull'holdout del modello rilasciato, IID contro per sito: 0.001330 contro 0.001615 (t = -1.26, 4 gdl); Yeom 0.5011 contro 0.5001. Manca il braccio con DP.</t>
+          <t>Braccio senza DP eseguito. Loss sull'holdout del modello rilasciato, IID contro per sito: 0.001330 contro 0.001615 (t = -1.26, 4 gdl); Yeom 0.5011 contro 0.5001. Con DP (eps = 64, C = 1): loss sull'holdout IID contro per sito 0.009363 contro 0.006326 (t = 1.03); attacchi al caso in entrambi.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>IID e per sito al punto operativo client-level: 2 celle x 5 seed = 10 run; la cella per sito coincide con quella di RQ1 al punto operativo.</t>
+          <t>Nessuna run mancante per il confronto minimo della guida.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>274 run totali</t>
+          <t>275 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -922,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F182"/>
+  <dimension ref="A1:F185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5050,12 +5050,12 @@
     <row r="159" ht="18" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
@@ -5067,21 +5067,21 @@
         <v>10</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.001742</v>
       </c>
       <c r="F159" s="3" t="n">
-        <v>25200</v>
+        <v>25239</v>
       </c>
     </row>
     <row r="160" ht="18" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -5093,21 +5093,21 @@
         <v>10</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.001963</v>
       </c>
       <c r="F160" s="3" t="n">
-        <v>26829</v>
+        <v>26781</v>
       </c>
     </row>
     <row r="161" ht="18" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
@@ -5119,21 +5119,21 @@
         <v>10</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.005474</v>
       </c>
       <c r="F161" s="3" t="n">
-        <v>1341</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -5145,7 +5145,7 @@
         <v>10</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.367252</v>
       </c>
       <c r="F162" s="3" t="n">
         <v>25200</v>
@@ -5154,12 +5154,12 @@
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
@@ -5171,7 +5171,7 @@
         <v>10</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.377587</v>
       </c>
       <c r="F163" s="3" t="n">
         <v>26829</v>
@@ -5180,12 +5180,12 @@
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -5197,7 +5197,7 @@
         <v>10</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.369278</v>
       </c>
       <c r="F164" s="3" t="n">
         <v>1341</v>
@@ -5206,12 +5206,12 @@
     <row r="165" ht="18" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -5223,7 +5223,7 @@
         <v>10</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.195433</v>
       </c>
       <c r="F165" s="3" t="n">
         <v>25200</v>
@@ -5232,12 +5232,12 @@
     <row r="166" ht="18" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -5249,7 +5249,7 @@
         <v>10</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.223175</v>
       </c>
       <c r="F166" s="3" t="n">
         <v>26829</v>
@@ -5258,12 +5258,12 @@
     <row r="167" ht="18" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
@@ -5275,7 +5275,7 @@
         <v>10</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.353804</v>
       </c>
       <c r="F167" s="3" t="n">
         <v>1341</v>
@@ -5284,7 +5284,7 @@
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -5298,10 +5298,10 @@
         </is>
       </c>
       <c r="D168" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F168" s="3" t="n">
         <v>25200</v>
@@ -5310,7 +5310,7 @@
     <row r="169" ht="18" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -5324,10 +5324,10 @@
         </is>
       </c>
       <c r="D169" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F169" s="3" t="n">
         <v>26829</v>
@@ -5336,7 +5336,7 @@
     <row r="170" ht="18" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -5350,10 +5350,10 @@
         </is>
       </c>
       <c r="D170" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F170" s="3" t="n">
         <v>1341</v>
@@ -5362,7 +5362,7 @@
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -5388,7 +5388,7 @@
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -5414,7 +5414,7 @@
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -5440,12 +5440,12 @@
     <row r="174" ht="18" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -5457,7 +5457,7 @@
         <v>3</v>
       </c>
       <c r="E174" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F174" s="3" t="n">
         <v>25200</v>
@@ -5466,12 +5466,12 @@
     <row r="175" ht="18" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
@@ -5483,7 +5483,7 @@
         <v>3</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F175" s="3" t="n">
         <v>26829</v>
@@ -5492,12 +5492,12 @@
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -5509,7 +5509,7 @@
         <v>3</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F176" s="3" t="n">
         <v>1341</v>
@@ -5518,12 +5518,12 @@
     <row r="177" ht="18" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
@@ -5535,7 +5535,7 @@
         <v>3</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F177" s="3" t="n">
         <v>25200</v>
@@ -5544,12 +5544,12 @@
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -5561,7 +5561,7 @@
         <v>3</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F178" s="3" t="n">
         <v>26829</v>
@@ -5570,12 +5570,12 @@
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
@@ -5587,7 +5587,7 @@
         <v>3</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.120528</v>
       </c>
       <c r="F179" s="3" t="n">
         <v>1341</v>
@@ -5596,7 +5596,7 @@
     <row r="180" ht="18" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -5622,7 +5622,7 @@
     <row r="181" ht="18" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
     <row r="182" ht="18" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -5668,6 +5668,84 @@
         <v>0.006995</v>
       </c>
       <c r="F182" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="183" ht="18" customHeight="1">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E183" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F183" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="184" ht="18" customHeight="1">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E184" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F184" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="185" ht="18" customHeight="1">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E185" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F185" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -6597,7 +6675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7255,8 +7333,110 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="13" ht="76" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>rq2-per_site-eps64</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>497</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>289.33</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>16.41</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>12.653</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>11.557</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.623</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0.1803</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>1.648</v>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="76" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>rq2-iid-eps64</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>346</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>289.35</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>3.444</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>9.984999999999999</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>-4.605</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.1919</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.2226</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>1.648</v>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>
@@ -7273,7 +7453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8138,6 +8318,999 @@
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="3" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>CON DP: dp-fedavg, eps = 64 per round, C = 1 (stesso punto per le due partizioni, scelto prima di vederle), 5 seed per braccio</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>per sito, media</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>IID, media</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>differenza appaiata IID - per sito</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>deviazione standard</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>t (4 gdl)</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>seed con IID sotto per sito</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>lettura</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.006326</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.009363</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>0.003037</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0.006619</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0.006026</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>0.009051999999999999</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0.003026</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0.006661</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0.000299</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.000311</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1.1e-05</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>1 su 5</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0.002659</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>0.002689</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>3e-05</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>9.8e-05</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>1 su 5</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.499028</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0.50135</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0.002323</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0.004817</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>1 su 5</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0.500522</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>0.500304</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>-0.000218</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0.001149</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0.501376</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0.501047</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>-0.000329</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.001153</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0.501488</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>0.499703</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>-0.001785</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0.005406</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0.01087</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>0.008215999999999999</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>-0.002655</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0.001531</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>-3.88</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>5 su 5</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>il caso vale 0.01; differenza significativa</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>braccio (con DP)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>0.003937</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>0.003643</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>0.000294</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>0.002726</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>0.499613</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>0.499224</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>0.499645</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0.501071</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>0.012444</v>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>0.009967</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0.009642</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0.000324</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0.002783</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0.503247</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>0.499196</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>0.499985</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0.494312</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>0.008994</v>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>0.004995</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>0.004636</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>0.000359</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0.002749</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0.497099</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0.5001</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>0.501649</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>0.502277</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>0.010943</v>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>0.004987</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>0.004625</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0.000362</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0.002783</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>0.502647</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0.499491</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>0.501643</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0.500728</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>0.007346</v>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>0.006151</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>0.005983</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>0.000168</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>0.002117</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>0.508148</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>0.502789</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>0.502968</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>0.503597</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>0.011022</v>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>0.019347</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>0.019246</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>0.000102</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>0.001997</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>0.5024650000000001</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>0.500958</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>0.500699</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0.510864</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>0.010644</v>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>0.011394</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>0.011192</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>0.000202</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0.002881</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>0.492682</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0.499263</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>0.500626</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0.50064</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>0.011621</v>
+      </c>
+    </row>
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>0.00821</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>0.007937</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>0.000273</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0.002906</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>0.499042</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0.500602</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0.5012990000000001</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0.49605</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>0.007572</v>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>0.005152</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>0.004678</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>0.000474</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0.002822</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>0.497597</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0.501236</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>0.5019940000000001</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>0.499856</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>0.008321</v>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>0.004303</v>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>0.00381</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>0.0004929999999999999</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0.002976</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>0.499351</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0.501273</v>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>0.50161</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0.49656</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>0.006522</v>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Fonte: experiments_altre_macchine/rq2-per_site-eps64 e rq2-iid-eps64 (seconda macchina, commit 3d4d318). Molteplicita': 18 test appaiati in questo foglio, 1 con |t| &gt; 2.776; a alpha = 0.05 senza correzione ce ne si attende circa 0.9 per caso. Metriche primarie (ESPERIMENTI.md, sezione 0): loss sull'holdout per il costo, Yeom e test per record (foglio Worst_case_per_record) per l'attacco; LiRA e Shadow sono secondarie e la calibrazione di LiRA e' degenere (STATO.md 3.4).</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n"/>
+      <c r="C49" s="3" t="n"/>
+      <c r="D49" s="3" t="n"/>
+      <c r="E49" s="3" t="n"/>
+      <c r="F49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="n"/>
+      <c r="I49" s="3" t="n"/>
+      <c r="J49" s="3" t="n"/>
+      <c r="K49" s="3" t="n"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="3" t="n"/>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
+      <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
+      <c r="I50" s="3" t="n"/>
+      <c r="J50" s="3" t="n"/>
+      <c r="K50" s="3" t="n"/>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>COSTO DELLA DP PER PARTIZIONE: loss sull'holdout con DP / senza DP, stesso seed</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n"/>
+      <c r="C51" s="3" t="n"/>
+      <c r="D51" s="3" t="n"/>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n"/>
+      <c r="G51" s="3" t="n"/>
+      <c r="H51" s="3" t="n"/>
+      <c r="I51" s="3" t="n"/>
+      <c r="J51" s="3" t="n"/>
+      <c r="K51" s="3" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>456</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>789</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>media geometrica</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n"/>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+      <c r="K52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>per sito</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="H53" s="3" t="n"/>
+      <c r="I53" s="3" t="n"/>
+      <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>IID</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>15.03</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="H54" s="3" t="n"/>
+      <c r="I54" s="3" t="n"/>
+      <c r="J54" s="3" t="n"/>
+      <c r="K54" s="3" t="n"/>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Interazione partizione x DP, sul logaritmo del rapporto (IID - per sito): media +0.450, sd 0.445, t(4) = 2.26; non significativa a 5 seed (|t| &lt; 2.776). Rapporto IID/per sito delle medie geometriche: 1.57.</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
+      <c r="I55" s="3" t="n"/>
+      <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
E-B: seed 456 di sigma=1; registro delle run corretto per record-DP, mu=0 e altre macchine (seg 56); -dirty del seed 456 (seg 57); SprintLog 10zz+136
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -562,7 +562,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>172 run in regime naturale</t>
+          <t>192 run in regime naturale</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>275 run totali</t>
+          <t>297 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
E-B: sigma=1 completa a 5 seed (1.4 volte il no-DP, attacchi al caso, z=0.18); cella record-DP in Utility_privacy_limite e C15; righe RQ1/RQ3 dai dati (seg 56); seg 58; SprintLog 10zz+137
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -562,7 +562,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>192 run in regime naturale</t>
+          <t>192 run in regime naturale, 5 record-DP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>C01..C11</t>
+          <t>C01..C15</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Nessuna lacuna sul fattore DP. Manca il braccio B1 'clipping senza rumore' (sigma=0), che la guida chiede in Fase B per separare l'effetto del clipping da quello del rumore.</t>
+          <t>Client-level: nessuna cella a 5 seed sotto 3 volte il no-DP sull'holdout del modello rilasciato; la migliore e' dp-fedavg, eps=64.0, 4.5 volte. Record-level: record-DP, nm=1.0, 5 seed, 1.4 volte. Mancano il braccio B1 'clipping senza rumore' (sigma=0, segnalazione 38) e la cella no-DP con GroupNorm, che separa rumore e architettura nelle celle record-DP.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>1 cella B1: clipping attivo, sigma=0, stessi 5 seed della cella di riferimento. Riusa i config esistenti cambiando un solo parametro.</t>
+          <t>B1: 1 cella x 5 seed, dopo il flag --clip-only. Cella no-DP con GroupNorm: 5 seed. Altri livelli di sigma per E-B (ESPERIMENTI.md).</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -614,7 +614,7 @@
     <row r="3" ht="160" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>10 run E-D senza DP (seconda macchina)</t>
+          <t>20 run E-D, senza DP e con DP (seconda macchina)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Braccio senza DP eseguito. Loss sull'holdout del modello rilasciato, IID contro per sito: 0.001330 contro 0.001615 (t = -1.26, 4 gdl); Yeom 0.5011 contro 0.5001. Con DP (eps = 64, C = 1): loss sull'holdout IID contro per sito 0.009363 contro 0.006326 (t = 1.03); attacchi al caso in entrambi.</t>
+          <t>Bracci senza DP e con DP eseguiti. Senza DP, loss sull'holdout del modello rilasciato, IID contro per sito: 0.001330 contro 0.001615 (t = -1.26, 4 gdl); Yeom 0.5011 contro 0.5001. Con DP (eps = 64, C = 1): loss sull'holdout IID contro per sito 0.009363 contro 0.006326 (t = 1.03); attacchi al caso in entrambi.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>297 run totali</t>
+          <t>300 run totali</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>lacuna strutturale</t>
+          <t>lacuna da colmare con E-E</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -691,12 +691,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>proximal_mu = 0.01 su 235 run su 235. Nessuna esecuzione con mu=0, quindi il confronto FedAvg/FedProx non e' recuperabile dai dati esistenti.</t>
+          <t>Nessuna run con mu = 0 in questo checkout (300 run nel registro). E-E gira su un'altra macchina (ESPERIMENTI.md); il config del braccio con DP, experiment_rq3_mu0_eps64.yaml, e' pronto.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Ripetere la configurazione di Fase B con mu=0, appaiata per split e seed: 1 algoritmo x 2 livelli di protezione x 5 seed = 10 run.</t>
+          <t>E-E: mu = 0 e mu = 0.01, senza DP e a eps = 64 con C = 1, 5 seed, tutte sulla stessa macchina (segnalazione 55): 20 run.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -5760,7 +5760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6664,6 +6664,58 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>record-DP, nm=1.0</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.002178</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.001797</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0.5007</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.5022</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0.5006</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0.009599999999999999</v>
+      </c>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="n">
+        <v>30.45</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 30.5; con lo shuffle il limite valido e' 1212. Non e' confrontabile con l'eps per round del client-level. Il rapporto di costo mescola rumore e GroupNorm (manca la cella no-DP con GroupNorm). Bound VACUO come nelle celle client-level.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6675,7 +6727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7435,8 +7487,59 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="15" ht="76" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>recordDP_nm1</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>17389</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>415</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>288.95</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>7.207</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>9.388</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>-1.102</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0.2215</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>0.183</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>2.387</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>1.662</v>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>

</xml_diff>

<commit_message>
RQ3 nelle matrici: foglio RQ3_algoritmo (appaiato FedAvg-FedProx, curva per round), C-RQ3 e sintesi dai dati; seg 59 nel glossario; SprintLog 10zz+140
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -13,7 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utility_privacy_limite" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worst_case_per_record" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RQ2_partizione" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossario_metriche" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RQ3_algoritmo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossario_metriche" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrice_sintesi'!$A$1:$I$1</definedName>
@@ -562,7 +563,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>192 run in regime naturale, 5 record-DP</t>
+          <t>202 run in regime naturale, 8 record-DP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -577,7 +578,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>C01..C15</t>
+          <t>C01..C16</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -587,7 +588,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Client-level: nessuna cella a 5 seed sotto 3 volte il no-DP sull'holdout del modello rilasciato; la migliore e' dp-fedavg, eps=64.0, 4.5 volte. Record-level: record-DP, nm=1.0, 5 seed, 1.4 volte. Mancano il braccio B1 'clipping senza rumore' (sigma=0, segnalazione 38) e la cella no-DP con GroupNorm, che separa rumore e architettura nelle celle record-DP.</t>
+          <t>Client-level: nessuna cella a 5 seed sotto 3 volte il no-DP sull'holdout del modello rilasciato; la migliore e' dp-fedavg, eps=64.0, 4.5 volte. Record-level: record-DP, nm=1.0, 5 seed, 1.4 volte; record-DP, nm=2.0, 3 seed, 1.4 volte. Mancano il braccio B1 'clipping senza rumore' (sigma=0, segnalazione 38) e la cella no-DP con GroupNorm, che separa rumore e architettura nelle celle record-DP.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -666,7 +667,7 @@
     <row r="4" ht="160" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>300 run totali</t>
+          <t>10 run E-E senza DP (terza macchina)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -674,9 +675,9 @@
           <t>RQ3</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>lacuna da colmare con E-E</t>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>completata da verificare</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -686,17 +687,17 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>si, appaiando per seed</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Nessuna run con mu = 0 in questo checkout (300 run nel registro). E-E gira su un'altra macchina (ESPERIMENTI.md); il config del braccio con DP, experiment_rq3_mu0_eps64.yaml, e' pronto.</t>
+          <t>Senza DP, loss sull'holdout del modello rilasciato, FedAvg contro FedProx: 0.000397 contro 0.001564 (t = -6.63, 4 gdl); Yeom 0.5011 contro 0.5000. Braccio con DP (eps = 64, C = 1) in corso.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>E-E: mu = 0 e mu = 0.01, senza DP e a eps = 64 con C = 1, 5 seed, tutte sulla stessa macchina (segnalazione 55): 20 run.</t>
+          <t>Braccio con DP: 2 algoritmi x 5 seed = 10 run sulla stessa macchina. Prove su mu a un seed (ESPERIMENTI.md, E-E).</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -706,7 +707,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Attenzione: proximal_mu vive in cfg['ml'], non in cfg['experiment']. Impostarlo nel posto sbagliato verrebbe ignorato in silenzio.</t>
+          <t>Tutta la campagna usa FedProx mu = 0.01 come base: se cambiarla e' una decisione del supervisore. La loss locale di FedProx include il termine prossimale (segnalazione 59).</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -922,7 +923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F185"/>
+  <dimension ref="A1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5128,12 +5129,12 @@
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -5145,7 +5146,7 @@
         <v>10</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.002036</v>
       </c>
       <c r="F162" s="3" t="n">
         <v>25200</v>
@@ -5154,12 +5155,12 @@
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
@@ -5171,7 +5172,7 @@
         <v>10</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.002171</v>
       </c>
       <c r="F163" s="3" t="n">
         <v>26829</v>
@@ -5180,12 +5181,12 @@
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -5197,7 +5198,7 @@
         <v>10</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.005838</v>
       </c>
       <c r="F164" s="3" t="n">
         <v>1341</v>
@@ -5206,12 +5207,12 @@
     <row r="165" ht="18" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -5223,7 +5224,7 @@
         <v>10</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.367252</v>
       </c>
       <c r="F165" s="3" t="n">
         <v>25200</v>
@@ -5232,12 +5233,12 @@
     <row r="166" ht="18" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -5249,7 +5250,7 @@
         <v>10</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.377587</v>
       </c>
       <c r="F166" s="3" t="n">
         <v>26829</v>
@@ -5258,12 +5259,12 @@
     <row r="167" ht="18" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
@@ -5275,7 +5276,7 @@
         <v>10</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.369278</v>
       </c>
       <c r="F167" s="3" t="n">
         <v>1341</v>
@@ -5284,12 +5285,12 @@
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -5301,7 +5302,7 @@
         <v>10</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.195433</v>
       </c>
       <c r="F168" s="3" t="n">
         <v>25200</v>
@@ -5310,12 +5311,12 @@
     <row r="169" ht="18" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
@@ -5327,7 +5328,7 @@
         <v>10</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.223175</v>
       </c>
       <c r="F169" s="3" t="n">
         <v>26829</v>
@@ -5336,12 +5337,12 @@
     <row r="170" ht="18" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -5353,7 +5354,7 @@
         <v>10</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.353804</v>
       </c>
       <c r="F170" s="3" t="n">
         <v>1341</v>
@@ -5362,7 +5363,7 @@
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -5376,10 +5377,10 @@
         </is>
       </c>
       <c r="D171" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F171" s="3" t="n">
         <v>25200</v>
@@ -5388,7 +5389,7 @@
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -5402,10 +5403,10 @@
         </is>
       </c>
       <c r="D172" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F172" s="3" t="n">
         <v>26829</v>
@@ -5414,7 +5415,7 @@
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -5428,10 +5429,10 @@
         </is>
       </c>
       <c r="D173" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F173" s="3" t="n">
         <v>1341</v>
@@ -5440,7 +5441,7 @@
     <row r="174" ht="18" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -5466,7 +5467,7 @@
     <row r="175" ht="18" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -5492,7 +5493,7 @@
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -5518,12 +5519,12 @@
     <row r="177" ht="18" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
@@ -5535,7 +5536,7 @@
         <v>3</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F177" s="3" t="n">
         <v>25200</v>
@@ -5544,12 +5545,12 @@
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -5561,7 +5562,7 @@
         <v>3</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F178" s="3" t="n">
         <v>26829</v>
@@ -5570,12 +5571,12 @@
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
@@ -5587,7 +5588,7 @@
         <v>3</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F179" s="3" t="n">
         <v>1341</v>
@@ -5596,12 +5597,12 @@
     <row r="180" ht="18" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
@@ -5613,7 +5614,7 @@
         <v>3</v>
       </c>
       <c r="E180" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F180" s="3" t="n">
         <v>25200</v>
@@ -5622,12 +5623,12 @@
     <row r="181" ht="18" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
@@ -5639,7 +5640,7 @@
         <v>3</v>
       </c>
       <c r="E181" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F181" s="3" t="n">
         <v>26829</v>
@@ -5648,12 +5649,12 @@
     <row r="182" ht="18" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
@@ -5665,7 +5666,7 @@
         <v>3</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.120528</v>
       </c>
       <c r="F182" s="3" t="n">
         <v>1341</v>
@@ -5674,7 +5675,7 @@
     <row r="183" ht="18" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -5700,7 +5701,7 @@
     <row r="184" ht="18" customHeight="1">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -5726,7 +5727,7 @@
     <row r="185" ht="18" customHeight="1">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-nodp.log</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -5746,6 +5747,84 @@
         <v>0.006995</v>
       </c>
       <c r="F185" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="186" ht="18" customHeight="1">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E186" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F186" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="187" ht="18" customHeight="1">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E187" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F187" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="188" ht="18" customHeight="1">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E188" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F188" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -5760,7 +5839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6713,6 +6792,58 @@
       <c r="P17" s="3" t="inlineStr">
         <is>
           <t>UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 30.5; con lo shuffle il limite valido e' 1212. Non e' confrontabile con l'eps per round del client-level. Il rapporto di costo mescola rumore e GroupNorm (manca la cella no-DP con GroupNorm). Bound VACUO come nelle celle client-level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>record-DP, nm=2.0</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.002248</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.001873</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.4995</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.5006</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.4985</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.4974</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.0103</v>
+      </c>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>0.999881</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>0.9999400000000001</v>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 9.7; con lo shuffle il limite valido e' 355. Non e' confrontabile con l'eps per round del client-level. Il rapporto di costo mescola rumore e GroupNorm (manca la cella no-DP con GroupNorm). Bound VACUO come nelle celle client-level.</t>
         </is>
       </c>
     </row>
@@ -9426,6 +9557,1105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>metrica</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FedProx mu = 0.01, media (5 seed)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FedAvg mu = 0, media</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>differenza appaiata FedAvg - FedProx</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>deviazione standard</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>t (4 gdl)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>seed con FedAvg sotto FedProx</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>lettura</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>0.001564</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.000397</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>-0.001167</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.000394</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>-6.63</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>5 su 5</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.000185</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>-0.001115</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.000387</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>-6.44</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>5 su 5</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.000265</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.000213</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>-5.2e-05</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>7.2e-05</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>nessuna differenza significativa a 5 seed (|t| &lt; 2.776)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0.00168</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.000265</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>-0.001414</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.000387</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>-8.18</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>5 su 5</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>non confrontabile fra i bracci: con FedProx include il termine prossimale (segnalazione 59)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.500009</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.501142</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.001133</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.002514</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2 su 5</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0.5002180000000001</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.5003919999999999</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.000174</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.001597</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2 su 5</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0.501363</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.499479</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>-0.001884</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.003452</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>3 su 5</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0.501513</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.500846</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>-0.0006669999999999999</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.003873</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>4 su 5</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>entrambi i bracci al caso; nessuna differenza significativa a 5 seed</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.01033</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.01054</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0.00021</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.001385</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>1 su 5</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>il caso vale 0.01; nessuna differenza significativa</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Rapporto FedProx / FedAvg sulla loss sull'holdout per seed: 3.91, 3.85, 3.67, 3.68, 4.45; media geometrica 3.90.</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>braccio</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>loss holdout del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>loss sui membri del modello rilasciato</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>divario holdout - membri</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>loss addestramento locale (diagnostica)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC all'ultimo round</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Yeom, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Shadow, AUC media sui round</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, AUC</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>LiRA composto, TPR a FPR 1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>FedProx</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.001753</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.001545</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.000209</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.001886</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.496352</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0.496407</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.496827</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.503803</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0.011844</v>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>FedAvg</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.000449</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.00019</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.000259</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0.00028</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0.50185</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0.498965</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.499537</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.5011409999999999</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0.01012</v>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>FedProx</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.001872</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.001488</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.000383</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.00193</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.497536</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.498907</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.501413</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.502175</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0.008994</v>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>FedAvg</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.000486</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0.000183</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.000303</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0.000281</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0.497333</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.499451</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.499235</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0.501229</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0.009219</v>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>FedProx</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.000686</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.00062</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>6.600000000000001e-05</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.000963</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.501678</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.501206</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.503152</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0.499601</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0.011247</v>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>FedAvg</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.000187</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0.000176</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0.000227</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.501006</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.5001949999999999</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.496976</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0.494877</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0.011247</v>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>FedProx</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.001586</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.001316</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.000269</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.001711</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.503563</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0.50382</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.502298</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0.5017779999999999</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0.008772</v>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>789</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>FedAvg</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>0.000431</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0.000193</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0.000238</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0.000257</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0.5045500000000001</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0.504144</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0.502418</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0.501158</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0.010946</v>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>FedProx</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.001926</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.001529</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.000397</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.001908</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.500915</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0.5007470000000001</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>0.503124</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>0.50021</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>0.010795</v>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>FedAvg</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0.000433</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0.000181</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0.000252</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0.000283</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0.50097</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0.499203</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>0.499228</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>0.505826</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>0.011169</v>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="3" t="n"/>
+      <c r="B24" s="3" t="n"/>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>round</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>loss sull'holdout del modello globale, FedProx (media sui seed)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>idem, FedAvg</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.047995</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.047995</v>
+      </c>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0.003774</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>0.00423</v>
+      </c>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.002758</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.001101</v>
+      </c>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0.002432</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>0.000807</v>
+      </c>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0.002213</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.000652</v>
+      </c>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0.002068</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>0.000593</v>
+      </c>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="3" t="n"/>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0.00196</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0.0004929999999999999</v>
+      </c>
+      <c r="D32" s="3" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
+      <c r="J32" s="3" t="n"/>
+      <c r="K32" s="3" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0.001804</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>0.000499</v>
+      </c>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0.001679</v>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0.000391</v>
+      </c>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="3" t="n"/>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0.001564</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>0.000397</v>
+      </c>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="3" t="n"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="3" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Fonte: experiments_altre_macchine/rq3-mu0.01 e rq3-mu0 (E-E, senza DP, terza macchina, commit 478d471; i due bracci hanno girato in parallelo). Differiscono solo per ml.proximal_mu e sono appaiati per seed; il round 1 e' identico nei due bracci, perche' il termine prossimale entra dal round 2. Il braccio FedProx ha il config di nodp-sweep2 ma gira su un'altra macchina (segnalazione 55): il confronto usa i due bracci della stessa macchina.</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9584,7 +10814,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>NON e' la qualita' del modello rilasciato. Senza DP coincide quasi con la loss sull'holdout; con DP client-level misura quanto bene un client riadatta localmente il modello rumoroso che riceve, e la distanza dalla loss sull'holdout misura il danno del rumore aggiunto all'aggregazione.</t>
+          <t>NON e' la qualita' del modello rilasciato. Senza DP coincide quasi con la loss sull'holdout; con DP client-level misura quanto bene un client riadatta localmente il modello rumoroso che riceve, e la distanza dalla loss sull'holdout misura il danno del rumore aggiunto all'aggregazione. Con FedProx (mu &gt; 0) include il termine prossimale (mu/2)||w - w_globale||^2: fra celle con mu diversi non si confronta (segnalazione 59).</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
E-B: sigma=2 e no-DP GroupNorm a 5 seed, costo della DP per record 1.9 e 2.1 volte sul riferimento GroupNorm; E-E completo sul Mac con prove su mu; SprintLog 10zz+141
</commit_message>
<xml_diff>
--- a/risultati/Matrice_sintesi.xlsx
+++ b/risultati/Matrice_sintesi.xlsx
@@ -563,7 +563,7 @@
     <row r="2" ht="160" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>202 run in regime naturale, 8 record-DP</t>
+          <t>207 run in regime naturale, 10 record-DP</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>C01..C16</t>
+          <t>C01..C17</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Client-level: nessuna cella a 5 seed sotto 3 volte il no-DP sull'holdout del modello rilasciato; la migliore e' dp-fedavg, eps=64.0, 4.5 volte. Record-level: record-DP, nm=1.0, 5 seed, 1.4 volte; record-DP, nm=2.0, 3 seed, 1.4 volte. Mancano il braccio B1 'clipping senza rumore' (sigma=0, segnalazione 38) e la cella no-DP con GroupNorm, che separa rumore e architettura nelle celle record-DP.</t>
+          <t>Client-level: la migliore cella a 5 seed e' no-DP baseline, norm=group, 0.7 volte. Record-level: record-DP, nm=1.0, 5 seed, 1.4 volte; record-DP, nm=2.0, 5 seed, 1.6 volte. Mancano il braccio B1 'clipping senza rumore' (sigma=0, segnalazione 38) e la cella no-DP con GroupNorm, che separa rumore e architettura nelle celle record-DP.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -923,7 +923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F188"/>
+  <dimension ref="A1:F194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5051,7 +5051,7 @@
     <row r="159" ht="18" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm1.log</t>
+          <t>rq1_nodp_groupnorm.log</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -5068,16 +5068,16 @@
         <v>10</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>0.001742</v>
+        <v>0.000749</v>
       </c>
       <c r="F159" s="3" t="n">
-        <v>25239</v>
+        <v>25200</v>
       </c>
     </row>
     <row r="160" ht="18" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm1.log</t>
+          <t>rq1_nodp_groupnorm.log</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -5094,16 +5094,16 @@
         <v>10</v>
       </c>
       <c r="E160" s="3" t="n">
-        <v>0.001963</v>
+        <v>0.000757</v>
       </c>
       <c r="F160" s="3" t="n">
-        <v>26781</v>
+        <v>26829</v>
       </c>
     </row>
     <row r="161" ht="18" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm1.log</t>
+          <t>rq1_nodp_groupnorm.log</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -5120,16 +5120,16 @@
         <v>10</v>
       </c>
       <c r="E161" s="3" t="n">
-        <v>0.005474</v>
+        <v>0.001676</v>
       </c>
       <c r="F161" s="3" t="n">
-        <v>1350</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="162" ht="18" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm2.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -5146,16 +5146,16 @@
         <v>10</v>
       </c>
       <c r="E162" s="3" t="n">
-        <v>0.002036</v>
+        <v>0.001742</v>
       </c>
       <c r="F162" s="3" t="n">
-        <v>25200</v>
+        <v>25239</v>
       </c>
     </row>
     <row r="163" ht="18" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm2.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -5172,16 +5172,16 @@
         <v>10</v>
       </c>
       <c r="E163" s="3" t="n">
-        <v>0.002171</v>
+        <v>0.001963</v>
       </c>
       <c r="F163" s="3" t="n">
-        <v>26829</v>
+        <v>26781</v>
       </c>
     </row>
     <row r="164" ht="18" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>rq1_recorddp_nm2.log</t>
+          <t>rq1_recorddp_nm1.log</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -5198,21 +5198,21 @@
         <v>10</v>
       </c>
       <c r="E164" s="3" t="n">
-        <v>0.005838</v>
+        <v>0.005474</v>
       </c>
       <c r="F164" s="3" t="n">
-        <v>1341</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="165" ht="18" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
@@ -5224,7 +5224,7 @@
         <v>10</v>
       </c>
       <c r="E165" s="3" t="n">
-        <v>0.367252</v>
+        <v>0.002036</v>
       </c>
       <c r="F165" s="3" t="n">
         <v>25200</v>
@@ -5233,12 +5233,12 @@
     <row r="166" ht="18" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -5250,7 +5250,7 @@
         <v>10</v>
       </c>
       <c r="E166" s="3" t="n">
-        <v>0.377587</v>
+        <v>0.002171</v>
       </c>
       <c r="F166" s="3" t="n">
         <v>26829</v>
@@ -5259,12 +5259,12 @@
     <row r="167" ht="18" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>stradaB_rerun.log</t>
+          <t>rq1_recorddp_nm2.log</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=0.1)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
@@ -5276,7 +5276,7 @@
         <v>10</v>
       </c>
       <c r="E167" s="3" t="n">
-        <v>0.369278</v>
+        <v>0.005838</v>
       </c>
       <c r="F167" s="3" t="n">
         <v>1341</v>
@@ -5285,12 +5285,12 @@
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq3_mac.log</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -5299,10 +5299,10 @@
         </is>
       </c>
       <c r="D168" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E168" s="3" t="n">
-        <v>0.195433</v>
+        <v>0.000394</v>
       </c>
       <c r="F168" s="3" t="n">
         <v>25200</v>
@@ -5311,12 +5311,12 @@
     <row r="169" ht="18" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq3_mac.log</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
@@ -5325,10 +5325,10 @@
         </is>
       </c>
       <c r="D169" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E169" s="3" t="n">
-        <v>0.223175</v>
+        <v>0.000342</v>
       </c>
       <c r="F169" s="3" t="n">
         <v>26829</v>
@@ -5337,12 +5337,12 @@
     <row r="170" ht="18" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-central.log</t>
+          <t>rq3_mac.log</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -5351,10 +5351,10 @@
         </is>
       </c>
       <c r="D170" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E170" s="3" t="n">
-        <v>0.353804</v>
+        <v>0.000572</v>
       </c>
       <c r="F170" s="3" t="n">
         <v>1341</v>
@@ -5363,12 +5363,12 @@
     <row r="171" ht="18" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
@@ -5380,7 +5380,7 @@
         <v>10</v>
       </c>
       <c r="E171" s="3" t="n">
-        <v>0.002174</v>
+        <v>0.367252</v>
       </c>
       <c r="F171" s="3" t="n">
         <v>25200</v>
@@ -5389,12 +5389,12 @@
     <row r="172" ht="18" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -5406,7 +5406,7 @@
         <v>10</v>
       </c>
       <c r="E172" s="3" t="n">
-        <v>0.002005</v>
+        <v>0.377587</v>
       </c>
       <c r="F172" s="3" t="n">
         <v>26829</v>
@@ -5415,12 +5415,12 @@
     <row r="173" ht="18" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>verify-10rounds-nodp.log</t>
+          <t>stradaB_rerun.log</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=0.1)</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
@@ -5432,7 +5432,7 @@
         <v>10</v>
       </c>
       <c r="E173" s="3" t="n">
-        <v>0.005707</v>
+        <v>0.369278</v>
       </c>
       <c r="F173" s="3" t="n">
         <v>1341</v>
@@ -5441,12 +5441,12 @@
     <row r="174" ht="18" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -5455,10 +5455,10 @@
         </is>
       </c>
       <c r="D174" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E174" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.195433</v>
       </c>
       <c r="F174" s="3" t="n">
         <v>25200</v>
@@ -5467,12 +5467,12 @@
     <row r="175" ht="18" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
@@ -5481,10 +5481,10 @@
         </is>
       </c>
       <c r="D175" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E175" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.223175</v>
       </c>
       <c r="F175" s="3" t="n">
         <v>26829</v>
@@ -5493,12 +5493,12 @@
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>verify-mu-anchor.log</t>
+          <t>verify-10rounds-central.log</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -5507,10 +5507,10 @@
         </is>
       </c>
       <c r="D176" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E176" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.353804</v>
       </c>
       <c r="F176" s="3" t="n">
         <v>1341</v>
@@ -5519,7 +5519,7 @@
     <row r="177" ht="18" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -5533,10 +5533,10 @@
         </is>
       </c>
       <c r="D177" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E177" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.002174</v>
       </c>
       <c r="F177" s="3" t="n">
         <v>25200</v>
@@ -5545,7 +5545,7 @@
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -5559,10 +5559,10 @@
         </is>
       </c>
       <c r="D178" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E178" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.002005</v>
       </c>
       <c r="F178" s="3" t="n">
         <v>26829</v>
@@ -5571,7 +5571,7 @@
     <row r="179" ht="18" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>verify-outlier-fix.log</t>
+          <t>verify-10rounds-nodp.log</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -5585,10 +5585,10 @@
         </is>
       </c>
       <c r="D179" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E179" s="3" t="n">
-        <v>0.006995</v>
+        <v>0.005707</v>
       </c>
       <c r="F179" s="3" t="n">
         <v>1341</v>
@@ -5597,12 +5597,12 @@
     <row r="180" ht="18" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
@@ -5614,7 +5614,7 @@
         <v>3</v>
       </c>
       <c r="E180" s="3" t="n">
-        <v>0.086894</v>
+        <v>0.003394</v>
       </c>
       <c r="F180" s="3" t="n">
         <v>25200</v>
@@ -5623,12 +5623,12 @@
     <row r="181" ht="18" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
@@ -5640,7 +5640,7 @@
         <v>3</v>
       </c>
       <c r="E181" s="3" t="n">
-        <v>0.076844</v>
+        <v>0.002953</v>
       </c>
       <c r="F181" s="3" t="n">
         <v>26829</v>
@@ -5649,12 +5649,12 @@
     <row r="182" ht="18" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-central.log</t>
+          <t>verify-mu-anchor.log</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>DP (eps=1.0)</t>
+          <t>no-DP</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
@@ -5666,7 +5666,7 @@
         <v>3</v>
       </c>
       <c r="E182" s="3" t="n">
-        <v>0.120528</v>
+        <v>0.006995</v>
       </c>
       <c r="F182" s="3" t="n">
         <v>1341</v>
@@ -5675,7 +5675,7 @@
     <row r="183" ht="18" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -5701,7 +5701,7 @@
     <row r="184" ht="18" customHeight="1">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -5727,7 +5727,7 @@
     <row r="185" ht="18" customHeight="1">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>verify-shadow-universe-nodp.log</t>
+          <t>verify-outlier-fix.log</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -5753,12 +5753,12 @@
     <row r="186" ht="18" customHeight="1">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
@@ -5770,7 +5770,7 @@
         <v>3</v>
       </c>
       <c r="E186" s="3" t="n">
-        <v>0.003394</v>
+        <v>0.086894</v>
       </c>
       <c r="F186" s="3" t="n">
         <v>25200</v>
@@ -5779,12 +5779,12 @@
     <row r="187" ht="18" customHeight="1">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
@@ -5796,7 +5796,7 @@
         <v>3</v>
       </c>
       <c r="E187" s="3" t="n">
-        <v>0.002953</v>
+        <v>0.076844</v>
       </c>
       <c r="F187" s="3" t="n">
         <v>26829</v>
@@ -5805,12 +5805,12 @@
     <row r="188" ht="18" customHeight="1">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>verify-sigma-fix.log</t>
+          <t>verify-shadow-universe-central.log</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>no-DP</t>
+          <t>DP (eps=1.0)</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -5822,9 +5822,165 @@
         <v>3</v>
       </c>
       <c r="E188" s="3" t="n">
+        <v>0.120528</v>
+      </c>
+      <c r="F188" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="189" ht="18" customHeight="1">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E189" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F189" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="190" ht="18" customHeight="1">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E190" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F190" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="191" ht="18" customHeight="1">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>verify-shadow-universe-nodp.log</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E191" s="3" t="n">
         <v>0.006995</v>
       </c>
-      <c r="F188" s="3" t="n">
+      <c r="F191" s="3" t="n">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="192" ht="18" customHeight="1">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>caltech</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E192" s="3" t="n">
+        <v>0.003394</v>
+      </c>
+      <c r="F192" s="3" t="n">
+        <v>25200</v>
+      </c>
+    </row>
+    <row r="193" ht="18" customHeight="1">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>jpl</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E193" s="3" t="n">
+        <v>0.002953</v>
+      </c>
+      <c r="F193" s="3" t="n">
+        <v>26829</v>
+      </c>
+    </row>
+    <row r="194" ht="18" customHeight="1">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>verify-sigma-fix.log</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>no-DP</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>office1</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E194" s="3" t="n">
+        <v>0.006995</v>
+      </c>
+      <c r="F194" s="3" t="n">
         <v>1341</v>
       </c>
     </row>
@@ -5839,7 +5995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6746,104 +6902,150 @@
     <row r="17" ht="80" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>record-DP, nm=1.0</t>
+          <t>no-DP baseline, norm=group</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
         <v>5</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.002178</v>
+        <v>0.001163</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.001797</v>
+        <v>0.000864</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="G17" s="3" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0.5012</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.5004999999999999</v>
+      </c>
+      <c r="J17" s="3" t="n">
         <v>0.5007</v>
       </c>
-      <c r="H17" s="3" t="n">
-        <v>0.5022</v>
-      </c>
-      <c r="I17" s="3" t="n">
-        <v>0.5004</v>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>0.5006</v>
-      </c>
       <c r="K17" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0094</v>
       </c>
       <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n">
-        <v>30.45</v>
-      </c>
-      <c r="N17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="n"/>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 30.5; con lo shuffle il limite valido e' 1212. Non e' confrontabile con l'eps per round del client-level. Il rapporto di costo mescola rumore e GroupNorm (manca la cella no-DP con GroupNorm). Bound VACUO come nelle celle client-level.</t>
+          <t>riferimento senza DP: nessuna garanzia da confrontare</t>
         </is>
       </c>
     </row>
     <row r="18" ht="80" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>record-DP, nm=2.0</t>
+          <t>record-DP, nm=1.0</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.002248</v>
+        <v>0.002178</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>1.4</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.001873</v>
+        <v>0.001797</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>1.1</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0.4995</v>
+        <v>0.5007</v>
       </c>
       <c r="H18" s="3" t="n">
+        <v>0.5022</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="J18" s="3" t="n">
         <v>0.5006</v>
       </c>
-      <c r="I18" s="3" t="n">
-        <v>0.4985</v>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>0.4974</v>
-      </c>
       <c r="K18" s="3" t="n">
-        <v>0.0103</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="n">
-        <v>9.73</v>
+        <v>30.45</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>0.999881</v>
+        <v>1</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>0.9999400000000001</v>
+        <v>1</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 9.7; con lo shuffle il limite valido e' 355. Non e' confrontabile con l'eps per round del client-level. Il rapporto di costo mescola rumore e GroupNorm (manca la cella no-DP con GroupNorm). Bound VACUO come nelle celle client-level.</t>
+          <t>1.87 volte il no-DP con GroupNorm, il riferimento con la stessa normalizzazione. UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 30.5; con lo shuffle il limite valido e' 1212. Non e' confrontabile con l'eps per round del client-level. Bound VACUO come nelle celle client-level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>record-DP, nm=2.0</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.002471</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.002002</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0.5019</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.4988</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0.4975</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>0.999879</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>0.999939</v>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>2.12 volte il no-DP con GroupNorm, il riferimento con la stessa normalizzazione. UNITA' PROTETTA RECORD: al posto di eps_tot c'e' l'eps per record di Poisson, massimo sui client e gia' composto sui round, in media 9.7; con lo shuffle il limite valido e' 355. Non e' confrontabile con l'eps per round del client-level. Bound VACUO come nelle celle client-level.</t>
         </is>
       </c>
     </row>
@@ -6858,7 +7060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7669,8 +7871,110 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="16" ht="76" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>recordDP_nm2</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>17346</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>455</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>286.01</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>15.85</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>10.664</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>-0.243</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>-0.1114</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0.2222</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>-0.501</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>2.623</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>1.649</v>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="76" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>no-DP_groupnorm</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>17561</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>458</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>289.94</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>10.116</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>1.186</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>-0.1998</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0.2206</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>-0.906</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>2.608</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>1.651</v>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>NESSUN SEGNALE DI APPARTENENZA PER RECORD (test appaiato). L'eccesso sui membri c'e' anche fra i non-membri: e' stabilita' del ranking dovuta al record. Se l'utility e' distrutta, l'assenza di segnale non prova che la DP protegga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>criterio: membro in &gt;= 2 seed, percentile medio &gt;= 90.0, percentile minimo &gt;= 75.0; livello di caso da 200 permutazioni dei percentili DENTRO ogni seed (conserva la distribuzione marginale, distrugge solo la corrispondenza fra seed). Lettura primaria: test appaiato (segnalazione 47); il conteggio sui membri da solo misura la stabilita' del ranking.</t>
         </is>

</xml_diff>